<commit_message>
Made initial pcb layout without wiring
</commit_message>
<xml_diff>
--- a/Schematics & PCB/parts_order.xlsx
+++ b/Schematics & PCB/parts_order.xlsx
@@ -76,6 +76,186 @@
     <t xml:space="preserve">4654-FCR7350B-ND </t>
   </si>
   <si>
+    <t xml:space="preserve">Cyan 2P Screw Terminal TB002-500-02BE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/same-sky-formerly-cui-devices/TB002-500-02BE/10064069 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">102-6145-ND</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Green 2P Screw Terminal 691137710002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/w%C3%BCrth-elektronik/691137710002/6644051 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">732-10955-ND</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Green 4P Screw Terminal 691137710004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/w%C3%BCrth-elektronik/691137710004/6644053 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">732-10957-ND</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Green 10mm LED WP813GD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/kingbright/WP813GD/3084264 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">754-1898-ND</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Right angle THT Switch 1-1825027-1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/te-connectivity-alcoswitch-switches/1-1825027-1/1632544 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">450-1658-ND</t>
+  </si>
+  <si>
+    <t xml:space="preserve">47uF Al Electrolytic Capacitor 860010372004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/w%C3%BCrth-elektronik/860010672004/5726903</t>
+  </si>
+  <si>
+    <t xml:space="preserve">732-8596-1-ND</t>
+  </si>
+  <si>
+    <t xml:space="preserve">100nF Ceramic Capacitor CL21B104KBCNNNC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/samsung-electro-mechanics/CL21B104KBCNNNC/3886661 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">1276-1003-1-ND</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10uF Ceramic Capacitor C2012X5R1V106K125AC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/tdk/C2012X5R1V106K125AC/3951654 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">445-14418-1-ND</t>
+  </si>
+  <si>
+    <t xml:space="preserve">47uF Ceramic Capacitor JMK212BBJ476MG-T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/taiyo-yuden/JMK212BBJ476MG-T/4970731 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">587-4280-1-ND</t>
+  </si>
+  <si>
+    <t xml:space="preserve">47pF Ceramic Capacitor GCM1885C2A470JA16J</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/murata-electronics/GCM1885C2A470JA16J/2591757 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">490-GCM1885C2A470JA16JCT-ND</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12pF Ceramic Capacitor KGM15ACG2A120JM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/kyocera-avx/KGM15ACG2A120JM/1598332 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">478-KGM15ACG2A120JMCT-ND</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10uH Shielded Inductor SRU1048-100Y</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/bourns-inc/SRU1048-100Y/2352907 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">118-SRU1048-100YCT-ND</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6.8uH Shielded Inductor SLF7045T-6R8M1R7-PF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/tdk/SLF7045T-6R8M1R7-PF/755381 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">445-2029-1-ND</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PMOS 100V 6.6A FQD8P10TM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/onsemi/FQD8P10TM/1054070 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">FQD8P10TMCT-ND</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DIODE ZENER 24V 300mW MM3Z24VT1G</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/onsemi/MM3Z24VT1G/661665 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">MM3Z24VT1GOSCT-ND</t>
+  </si>
+  <si>
+    <t xml:space="preserve">30.1kΩ Thick Film resistor CR0805-FX-3012ELF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/bourns-inc/CR0805-FX-3012ELF/3784840 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">CR0805-FX-3012ELFCT-ND</t>
+  </si>
+  <si>
+    <t xml:space="preserve">158kΩ Thick Film resistor CR0805-FX-1583ELF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/bourns-inc/CR0805-FX-1583ELF/3784668 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">118-CR0805-FX-1583ELFCT-ND</t>
+  </si>
+  <si>
+    <t xml:space="preserve">422k Thick Film resistor CRCW0805422KFKEA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/vishay-dale/CRCW0805422KFKEA/1175961 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">541-422KCCT-ND</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10k Thick film Resistor RMCF0805FT10K0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/stackpole-electronics-inc/RMCF0805FT10K0/1760676 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">RMCF0805FT10K0CT-ND</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1k Thick film Resistor RNCP0805FTD1K00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/stackpole-electronics-inc/RNCP0805FTD1K00/2240229 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">RNCP0805FTD1K00CT-ND</t>
+  </si>
+  <si>
     <t xml:space="preserve">0.169Ω 1W Thick film resistor RLC73PD2BR169FTD</t>
   </si>
   <si>
@@ -85,283 +265,13 @@
     <t xml:space="preserve">1712-RLC73PD2BR169FTDCT-ND</t>
   </si>
   <si>
-    <t xml:space="preserve">47uF Al Electrolytic Capacitor 860010372004</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/w%C3%BCrth-elektronik/860010672004/5726903</t>
-  </si>
-  <si>
-    <t xml:space="preserve">732-8596-1-ND</t>
-  </si>
-  <si>
-    <t xml:space="preserve">100nF Ceramic Capacitor CL21B104KBCNNNC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/samsung-electro-mechanics/CL21B104KBCNNNC/3886661 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">1276-1003-1-ND</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cyan 2P Screw Terminal TB002-500-02BE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/same-sky-formerly-cui-devices/TB002-500-02BE/10064069 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">102-6145-ND</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Green 2P Screw Terminal 691137710002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/w%C3%BCrth-elektronik/691137710002/6644051 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">732-10955-ND</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Green 4P Screw Terminal 691137710004</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/w%C3%BCrth-elektronik/691137710004/6644053 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">732-10957-ND</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10uF Ceramic Capacitor C2012X5R1V106K125AC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/tdk/C2012X5R1V106K125AC/3951654 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">445-14418-1-ND</t>
-  </si>
-  <si>
-    <t xml:space="preserve">47uF Ceramic Capacitor JMK212BBJ476MG-T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/taiyo-yuden/JMK212BBJ476MG-T/4970731 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">587-4280-1-ND</t>
-  </si>
-  <si>
-    <t xml:space="preserve">47pF Ceramic Capacitor GCM1885C2A470JA16J</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/murata-electronics/GCM1885C2A470JA16J/2591757 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">490-GCM1885C2A470JA16JCT-ND</t>
-  </si>
-  <si>
-    <t xml:space="preserve">12pF Ceramic Capacitor KGM15ACG2A120JM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/kyocera-avx/KGM15ACG2A120JM/1598332 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">478-KGM15ACG2A120JMCT-ND</t>
-  </si>
-  <si>
-    <t xml:space="preserve">30.1kΩ Thick Film resistor CR0805-FX-3012ELF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/bourns-inc/CR0805-FX-3012ELF/3784840 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">CR0805-FX-3012ELFCT-ND</t>
-  </si>
-  <si>
-    <t xml:space="preserve">158kΩ Thick Film resistor CR0805-FX-1583ELF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/bourns-inc/CR0805-FX-1583ELF/3784668 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">118-CR0805-FX-1583ELFCT-ND</t>
-  </si>
-  <si>
-    <t xml:space="preserve">422k Thick Film resistor CRCW0805422KFKEA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/vishay-dale/CRCW0805422KFKEA/1175961 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">541-422KCCT-ND</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10uH Shielded Inductor SRU1048-100Y</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/bourns-inc/SRU1048-100Y/2352907 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">118-SRU1048-100YCT-ND</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6.8uH Shielded Inductor SLF7045T-6R8M1R7-PF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/tdk/SLF7045T-6R8M1R7-PF/755381 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">445-2029-1-ND</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PMOS 100V 6.6A FQD8P10TM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/onsemi/FQD8P10TM/1054070 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">FQD8P10TMCT-ND</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DIODE ZENER 24V 300mW MM3Z24VT1G</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/onsemi/MM3Z24VT1G/661665 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">MM3Z24VT1GOSCT-ND</t>
-  </si>
-  <si>
     <t xml:space="preserve">10K LINEAR Potentiometer PDB181-B225K-103B</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/bourns-inc/PDB181-B225K-103B/6153329</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
+    <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/bourns-inc/PDB181-B225K-103B/6153329 </t>
   </si>
   <si>
     <t xml:space="preserve">PDB181-B225K-103B</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Green 10mm LED WP813GD</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/kingbright/WP813GD/3084264</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">754-1898-ND</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Right angle THT Switch 1-1825027-1</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/te-connectivity-alcoswitch-switches/1-1825027-1/1632544</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">450-1658-ND</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10k Thick film Resistor RMCF0805FT10K0</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/stackpole-electronics-inc/RMCF0805FT10K0/1760676</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">RMCF0805FT10K0CT-ND</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1k Thick film Resistor RNCP0805FTD1K00</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/stackpole-electronics-inc/RNCP0805FTD1K00/2240229</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">RNCP0805FTD1K00CT-ND</t>
   </si>
   <si>
     <t xml:space="preserve">TOTAL</t>
@@ -375,7 +285,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="[$$-1409]#,##0.00;[RED]\-[$$-1409]#,##0.00"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="7">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -406,13 +316,6 @@
     </font>
     <font>
       <sz val="12"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FF0000FF"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
@@ -467,7 +370,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -514,10 +417,6 @@
     </xf>
     <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -749,96 +648,100 @@
       </c>
     </row>
     <row r="7" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B7" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="E7" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" s="11" t="n">
+        <v>0.62</v>
+      </c>
       <c r="G7" s="4"/>
     </row>
     <row r="8" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="4" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E8" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F8" s="11" t="n">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
       <c r="G8" s="4"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="4" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="E9" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F9" s="11" t="n">
-        <v>0.18</v>
+        <v>1.34</v>
       </c>
       <c r="G9" s="4"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="4" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F10" s="11" t="n">
-        <v>0.18</v>
+        <v>0.6</v>
       </c>
       <c r="G10" s="4"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="4" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="E11" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F11" s="11" t="n">
-        <v>0.62</v>
+        <v>0.49</v>
       </c>
       <c r="G11" s="4"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="C12" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="E12" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F12" s="11" t="n">
-        <v>0.7</v>
-      </c>
+      <c r="B12" s="0"/>
+      <c r="C12" s="0"/>
+      <c r="D12" s="0"/>
+      <c r="E12" s="0"/>
       <c r="G12" s="4"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -855,7 +758,7 @@
         <v>1</v>
       </c>
       <c r="F13" s="11" t="n">
-        <v>1.34</v>
+        <v>0.18</v>
       </c>
       <c r="G13" s="4"/>
     </row>
@@ -870,10 +773,10 @@
         <v>38</v>
       </c>
       <c r="E14" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F14" s="11" t="n">
-        <v>0.86</v>
+        <v>0.18</v>
       </c>
       <c r="G14" s="4"/>
     </row>
@@ -891,7 +794,7 @@
         <v>2</v>
       </c>
       <c r="F15" s="11" t="n">
-        <v>0.57</v>
+        <v>0.86</v>
       </c>
       <c r="G15" s="4"/>
     </row>
@@ -906,10 +809,10 @@
         <v>44</v>
       </c>
       <c r="E16" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F16" s="11" t="n">
-        <v>0.18</v>
+        <v>0.57</v>
       </c>
       <c r="G16" s="4"/>
     </row>
@@ -942,7 +845,7 @@
         <v>50</v>
       </c>
       <c r="E18" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F18" s="11" t="n">
         <v>0.18</v>
@@ -963,7 +866,7 @@
         <v>1</v>
       </c>
       <c r="F19" s="11" t="n">
-        <v>0.18</v>
+        <v>1.7</v>
       </c>
       <c r="G19" s="4"/>
     </row>
@@ -981,7 +884,7 @@
         <v>1</v>
       </c>
       <c r="F20" s="11" t="n">
-        <v>0.18</v>
+        <v>1.43</v>
       </c>
       <c r="G20" s="4"/>
     </row>
@@ -999,7 +902,7 @@
         <v>1</v>
       </c>
       <c r="F21" s="11" t="n">
-        <v>1.7</v>
+        <v>2.46</v>
       </c>
       <c r="G21" s="4"/>
     </row>
@@ -1017,109 +920,98 @@
         <v>1</v>
       </c>
       <c r="F22" s="11" t="n">
-        <v>1.43</v>
+        <v>0.31</v>
       </c>
       <c r="G22" s="4"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="C23" s="10" t="s">
-        <v>64</v>
-      </c>
-      <c r="D23" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="E23" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F23" s="11" t="n">
-        <v>2.46</v>
-      </c>
+      <c r="B23" s="0"/>
+      <c r="C23" s="0"/>
+      <c r="D23" s="0"/>
+      <c r="E23" s="0"/>
       <c r="G23" s="4"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="4" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="E24" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F24" s="11" t="n">
-        <v>0.31</v>
+        <v>0.18</v>
       </c>
       <c r="G24" s="4"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="C25" s="12" t="s">
-        <v>70</v>
+        <v>66</v>
+      </c>
+      <c r="C25" s="10" t="s">
+        <v>67</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="E25" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F25" s="11" t="n">
-        <v>2.36</v>
+        <v>0.18</v>
       </c>
       <c r="G25" s="4"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="C26" s="12" t="s">
-        <v>73</v>
+        <v>69</v>
+      </c>
+      <c r="C26" s="10" t="s">
+        <v>70</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="E26" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F26" s="11" t="n">
-        <v>0.6</v>
+        <v>0.18</v>
       </c>
       <c r="G26" s="4"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="C27" s="12" t="s">
-        <v>76</v>
+        <v>72</v>
+      </c>
+      <c r="C27" s="10" t="s">
+        <v>73</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="E27" s="7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F27" s="11" t="n">
-        <v>0.49</v>
+        <v>0.18</v>
       </c>
       <c r="G27" s="4"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="C28" s="12" t="s">
-        <v>79</v>
+        <v>75</v>
+      </c>
+      <c r="C28" s="10" t="s">
+        <v>76</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="E28" s="7" t="n">
         <v>3</v>
@@ -1131,28 +1023,38 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C29" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="D29" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="E29" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F29" s="11" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="G29" s="4"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B30" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="C29" s="12" t="s">
+      <c r="C30" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="D29" s="4" t="s">
+      <c r="D30" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="E29" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="F29" s="11" t="n">
-        <v>0.18</v>
-      </c>
-      <c r="G29" s="4"/>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B30" s="4"/>
-      <c r="C30" s="4"/>
-      <c r="D30" s="4"/>
-      <c r="E30" s="7"/>
-      <c r="F30" s="11"/>
+      <c r="E30" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F30" s="11" t="n">
+        <v>2.36</v>
+      </c>
       <c r="G30" s="4"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1201,27 +1103,24 @@
       <c r="G35" s="4"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B36" s="4"/>
-      <c r="C36" s="4"/>
-      <c r="D36" s="4"/>
-      <c r="E36" s="7"/>
-      <c r="F36" s="11"/>
+      <c r="B36" s="0"/>
+      <c r="C36" s="0"/>
+      <c r="D36" s="0"/>
+      <c r="E36" s="0"/>
       <c r="G36" s="4"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B37" s="4"/>
-      <c r="C37" s="4"/>
-      <c r="D37" s="4"/>
-      <c r="E37" s="7"/>
-      <c r="F37" s="11"/>
+      <c r="B37" s="0"/>
+      <c r="C37" s="0"/>
+      <c r="D37" s="0"/>
+      <c r="E37" s="0"/>
       <c r="G37" s="4"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B38" s="4"/>
-      <c r="C38" s="4"/>
-      <c r="D38" s="4"/>
-      <c r="E38" s="7"/>
-      <c r="F38" s="11"/>
+      <c r="B38" s="0"/>
+      <c r="C38" s="0"/>
+      <c r="D38" s="0"/>
+      <c r="E38" s="0"/>
       <c r="G38" s="4"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1249,67 +1148,59 @@
       <c r="G41" s="4"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B42" s="4"/>
-      <c r="C42" s="4"/>
-      <c r="D42" s="4"/>
-      <c r="E42" s="7"/>
-      <c r="F42" s="11"/>
+      <c r="B42" s="0"/>
+      <c r="C42" s="0"/>
+      <c r="D42" s="0"/>
+      <c r="E42" s="0"/>
       <c r="G42" s="4"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B43" s="4"/>
-      <c r="C43" s="4"/>
-      <c r="D43" s="4"/>
-      <c r="E43" s="7"/>
-      <c r="F43" s="11"/>
+      <c r="B43" s="0"/>
+      <c r="C43" s="0"/>
+      <c r="D43" s="0"/>
+      <c r="E43" s="0"/>
       <c r="G43" s="4"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B44" s="4"/>
-      <c r="C44" s="4"/>
-      <c r="D44" s="4"/>
-      <c r="E44" s="7"/>
-      <c r="F44" s="11"/>
+      <c r="B44" s="0"/>
+      <c r="C44" s="0"/>
+      <c r="D44" s="0"/>
+      <c r="E44" s="0"/>
       <c r="G44" s="4"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B45" s="4"/>
-      <c r="C45" s="4"/>
-      <c r="D45" s="4"/>
-      <c r="E45" s="7"/>
-      <c r="F45" s="4"/>
+      <c r="B45" s="0"/>
+      <c r="C45" s="0"/>
+      <c r="D45" s="0"/>
+      <c r="E45" s="0"/>
       <c r="G45" s="4"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B46" s="4"/>
-      <c r="C46" s="4"/>
-      <c r="D46" s="4"/>
-      <c r="E46" s="7"/>
-      <c r="F46" s="4"/>
+      <c r="B46" s="0"/>
+      <c r="C46" s="0"/>
+      <c r="D46" s="0"/>
+      <c r="E46" s="0"/>
       <c r="G46" s="4"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B47" s="4"/>
-      <c r="C47" s="4"/>
-      <c r="D47" s="4"/>
-      <c r="E47" s="7"/>
-      <c r="F47" s="4"/>
+      <c r="B47" s="0"/>
+      <c r="C47" s="0"/>
+      <c r="D47" s="0"/>
+      <c r="E47" s="0"/>
       <c r="G47" s="4"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B48" s="4"/>
-      <c r="C48" s="4"/>
-      <c r="D48" s="4"/>
-      <c r="E48" s="7"/>
-      <c r="F48" s="4"/>
+      <c r="B48" s="0"/>
+      <c r="C48" s="0"/>
+      <c r="D48" s="0"/>
+      <c r="E48" s="0"/>
       <c r="G48" s="4"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B49" s="4"/>
-      <c r="C49" s="4"/>
-      <c r="D49" s="4"/>
-      <c r="E49" s="7"/>
-      <c r="F49" s="4"/>
+      <c r="B49" s="0"/>
+      <c r="C49" s="0"/>
+      <c r="D49" s="0"/>
+      <c r="E49" s="0"/>
       <c r="G49" s="4"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1454,28 +1345,28 @@
     <hyperlink ref="C4" r:id="rId2" display="https://www.digikey.co.nz/en/products/detail/texas-instruments/DRV8231DDAR/16184249 "/>
     <hyperlink ref="C5" r:id="rId3" display="https://www.digikey.co.nz/en/products/detail/cliff-electronic-components-ltd/FCR7350R/17729035  "/>
     <hyperlink ref="C6" r:id="rId4" display="https://www.digikey.co.nz/en/products/detail/cliff-electronic-components-ltd/FCR7350B/17729030  "/>
-    <hyperlink ref="C8" r:id="rId5" display="https://www.digikey.co.nz/en/products/detail/te-connectivity-passive-product/RLC73PD2BR169FTD/19238107 "/>
-    <hyperlink ref="C9" r:id="rId6" display="https://www.digikey.co.nz/en/products/detail/w%C3%BCrth-elektronik/860010672004/5726903"/>
-    <hyperlink ref="C10" r:id="rId7" display="https://www.digikey.co.nz/en/products/detail/samsung-electro-mechanics/CL21B104KBCNNNC/3886661 "/>
-    <hyperlink ref="C11" r:id="rId8" display="https://www.digikey.co.nz/en/products/detail/same-sky-formerly-cui-devices/TB002-500-02BE/10064069 "/>
-    <hyperlink ref="C12" r:id="rId9" display="https://www.digikey.co.nz/en/products/detail/w%C3%BCrth-elektronik/691137710002/6644051 "/>
-    <hyperlink ref="C13" r:id="rId10" display="https://www.digikey.co.nz/en/products/detail/w%C3%BCrth-elektronik/691137710004/6644053 "/>
-    <hyperlink ref="C14" r:id="rId11" display="https://www.digikey.co.nz/en/products/detail/tdk/C2012X5R1V106K125AC/3951654 "/>
-    <hyperlink ref="C15" r:id="rId12" display="https://www.digikey.co.nz/en/products/detail/taiyo-yuden/JMK212BBJ476MG-T/4970731 "/>
-    <hyperlink ref="C16" r:id="rId13" display="https://www.digikey.co.nz/en/products/detail/murata-electronics/GCM1885C2A470JA16J/2591757 "/>
-    <hyperlink ref="C17" r:id="rId14" display="https://www.digikey.co.nz/en/products/detail/kyocera-avx/KGM15ACG2A120JM/1598332 "/>
-    <hyperlink ref="C18" r:id="rId15" display="https://www.digikey.co.nz/en/products/detail/bourns-inc/CR0805-FX-3012ELF/3784840 "/>
-    <hyperlink ref="C19" r:id="rId16" display="https://www.digikey.co.nz/en/products/detail/bourns-inc/CR0805-FX-1583ELF/3784668 "/>
-    <hyperlink ref="C20" r:id="rId17" display="https://www.digikey.co.nz/en/products/detail/vishay-dale/CRCW0805422KFKEA/1175961 "/>
-    <hyperlink ref="C21" r:id="rId18" display="https://www.digikey.co.nz/en/products/detail/bourns-inc/SRU1048-100Y/2352907 "/>
-    <hyperlink ref="C22" r:id="rId19" display="https://www.digikey.co.nz/en/products/detail/tdk/SLF7045T-6R8M1R7-PF/755381 "/>
-    <hyperlink ref="C23" r:id="rId20" display="https://www.digikey.co.nz/en/products/detail/onsemi/FQD8P10TM/1054070 "/>
-    <hyperlink ref="C24" r:id="rId21" display="https://www.digikey.co.nz/en/products/detail/onsemi/MM3Z24VT1G/661665 "/>
-    <hyperlink ref="C25" r:id="rId22" display="https://www.digikey.co.nz/en/products/detail/bourns-inc/PDB181-B225K-103B/6153329"/>
-    <hyperlink ref="C26" r:id="rId23" display="https://www.digikey.co.nz/en/products/detail/kingbright/WP813GD/3084264"/>
-    <hyperlink ref="C27" r:id="rId24" display="https://www.digikey.co.nz/en/products/detail/te-connectivity-alcoswitch-switches/1-1825027-1/1632544"/>
-    <hyperlink ref="C28" r:id="rId25" display="https://www.digikey.co.nz/en/products/detail/stackpole-electronics-inc/RMCF0805FT10K0/1760676"/>
-    <hyperlink ref="C29" r:id="rId26" display="https://www.digikey.co.nz/en/products/detail/stackpole-electronics-inc/RNCP0805FTD1K00/2240229"/>
+    <hyperlink ref="C7" r:id="rId5" display="https://www.digikey.co.nz/en/products/detail/same-sky-formerly-cui-devices/TB002-500-02BE/10064069 "/>
+    <hyperlink ref="C8" r:id="rId6" display="https://www.digikey.co.nz/en/products/detail/w%C3%BCrth-elektronik/691137710002/6644051 "/>
+    <hyperlink ref="C9" r:id="rId7" display="https://www.digikey.co.nz/en/products/detail/w%C3%BCrth-elektronik/691137710004/6644053 "/>
+    <hyperlink ref="C10" r:id="rId8" display="https://www.digikey.co.nz/en/products/detail/kingbright/WP813GD/3084264 "/>
+    <hyperlink ref="C11" r:id="rId9" display="https://www.digikey.co.nz/en/products/detail/te-connectivity-alcoswitch-switches/1-1825027-1/1632544 "/>
+    <hyperlink ref="C13" r:id="rId10" display="https://www.digikey.co.nz/en/products/detail/w%C3%BCrth-elektronik/860010672004/5726903"/>
+    <hyperlink ref="C14" r:id="rId11" display="https://www.digikey.co.nz/en/products/detail/samsung-electro-mechanics/CL21B104KBCNNNC/3886661 "/>
+    <hyperlink ref="C15" r:id="rId12" display="https://www.digikey.co.nz/en/products/detail/tdk/C2012X5R1V106K125AC/3951654 "/>
+    <hyperlink ref="C16" r:id="rId13" display="https://www.digikey.co.nz/en/products/detail/taiyo-yuden/JMK212BBJ476MG-T/4970731 "/>
+    <hyperlink ref="C17" r:id="rId14" display="https://www.digikey.co.nz/en/products/detail/murata-electronics/GCM1885C2A470JA16J/2591757 "/>
+    <hyperlink ref="C18" r:id="rId15" display="https://www.digikey.co.nz/en/products/detail/kyocera-avx/KGM15ACG2A120JM/1598332 "/>
+    <hyperlink ref="C19" r:id="rId16" display="https://www.digikey.co.nz/en/products/detail/bourns-inc/SRU1048-100Y/2352907 "/>
+    <hyperlink ref="C20" r:id="rId17" display="https://www.digikey.co.nz/en/products/detail/tdk/SLF7045T-6R8M1R7-PF/755381 "/>
+    <hyperlink ref="C21" r:id="rId18" display="https://www.digikey.co.nz/en/products/detail/onsemi/FQD8P10TM/1054070 "/>
+    <hyperlink ref="C22" r:id="rId19" display="https://www.digikey.co.nz/en/products/detail/onsemi/MM3Z24VT1G/661665 "/>
+    <hyperlink ref="C24" r:id="rId20" display="https://www.digikey.co.nz/en/products/detail/bourns-inc/CR0805-FX-3012ELF/3784840 "/>
+    <hyperlink ref="C25" r:id="rId21" display="https://www.digikey.co.nz/en/products/detail/bourns-inc/CR0805-FX-1583ELF/3784668 "/>
+    <hyperlink ref="C26" r:id="rId22" display="https://www.digikey.co.nz/en/products/detail/vishay-dale/CRCW0805422KFKEA/1175961 "/>
+    <hyperlink ref="C27" r:id="rId23" display="https://www.digikey.co.nz/en/products/detail/stackpole-electronics-inc/RMCF0805FT10K0/1760676 "/>
+    <hyperlink ref="C28" r:id="rId24" display="https://www.digikey.co.nz/en/products/detail/stackpole-electronics-inc/RNCP0805FTD1K00/2240229 "/>
+    <hyperlink ref="C29" r:id="rId25" display="https://www.digikey.co.nz/en/products/detail/te-connectivity-passive-product/RLC73PD2BR169FTD/19238107 "/>
+    <hyperlink ref="C30" r:id="rId26" display="https://www.digikey.co.nz/en/products/detail/bourns-inc/PDB181-B225K-103B/6153329 "/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>

<commit_message>
Finished BOM and finalised PCB layout
</commit_message>
<xml_diff>
--- a/Schematics & PCB/parts_order.xlsx
+++ b/Schematics & PCB/parts_order.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="107">
   <si>
     <t xml:space="preserve">Component</t>
   </si>
@@ -124,6 +124,72 @@
     <t xml:space="preserve">450-1658-ND</t>
   </si>
   <si>
+    <t xml:space="preserve">Orange LED 2mA XZCM2MOK54WA-1VF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/sunled/XZCM2MOK54WA-1VF/15761908 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">1497-XZCM2MOK54WA-1VFCT-ND</t>
+  </si>
+  <si>
+    <t xml:space="preserve">White LED 5mA LW Q98G.01-R2T1-3K6L-1-5-R18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/ams-osram-ag/LW-Q98G-01-R2T1-3K6L-1-5-R18/21556497 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">475-LWQ98G.01-R2T1-3K6L-1CT-ND</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PMOS 100V 6.6A FQD8P10TM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/onsemi/FQD8P10TM/1054070 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">FQD8P10TMCT-ND</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DOUBLE CHECK THE AMOUNTS AND STUFF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PMOS 30V 4.3A DMP3056L-7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/diodes-incorporated/DMP3056L-7/5126843 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">DMP3056L-7DICT-ND</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NMOS 60 V 265mA NX138BKR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/nexperia-usa-inc/NX138BKR/5981270 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">1727-2662-1-ND</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NMOS 20 V 3A SLMT320V3CN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/shenzhen-slkormicro-semicon-co-ltd/SLMT320V3CN/29782446 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">5399-SLMT320V3CNCT-ND</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DIODE ZENER 24V 300mW MM3Z24VT1G</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/onsemi/MM3Z24VT1G/661665 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">MM3Z24VT1GOSCT-ND</t>
+  </si>
+  <si>
     <t xml:space="preserve">47uF Al Electrolytic Capacitor 860010372004</t>
   </si>
   <si>
@@ -151,9 +217,6 @@
     <t xml:space="preserve">445-14418-1-ND</t>
   </si>
   <si>
-    <t xml:space="preserve">DOUBLE CHECK THE AMOUNTS AND STUFF</t>
-  </si>
-  <si>
     <t xml:space="preserve">47pF Ceramic Capacitor GCM1885C2A470JA16J</t>
   </si>
   <si>
@@ -163,15 +226,6 @@
     <t xml:space="preserve">490-GCM1885C2A470JA16JCT-ND</t>
   </si>
   <si>
-    <t xml:space="preserve">12pF Ceramic Capacitor KGM15ACG2A120JM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/kyocera-avx/KGM15ACG2A120JM/1598332 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">478-KGM15ACG2A120JMCT-ND</t>
-  </si>
-  <si>
     <t xml:space="preserve">47uF Ceramic Capacitor JMK212BBJ476MG-T</t>
   </si>
   <si>
@@ -193,105 +247,6 @@
     <t xml:space="preserve">445-2029-1-ND</t>
   </si>
   <si>
-    <t xml:space="preserve">PMOS 100V 6.6A FQD8P10TM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/onsemi/FQD8P10TM/1054070 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">FQD8P10TMCT-ND</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DIODE ZENER 24V 300mW MM3Z24VT1G</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/onsemi/MM3Z24VT1G/661665 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">MM3Z24VT1GOSCT-ND</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PMOS 30V 4.3A DMP3056L-7</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/diodes-incorporated/DMP3056L-7/5126843</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">DMP3056L-7DICT-ND</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NMOS 60 V 265mA NX138BKR</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/nexperia-usa-inc/NX138BKR/5981270</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">1727-2662-1-ND</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NMOS 20 V 3A SLMT320V3CN</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/shenzhen-slkormicro-semicon-co-ltd/SLMT320V3CN/29782446</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">5399-SLMT320V3CNCT-ND</t>
-  </si>
-  <si>
     <t xml:space="preserve">30.1kΩ Thick Film resistor CR0805-FX-3012ELF</t>
   </si>
   <si>
@@ -310,15 +265,6 @@
     <t xml:space="preserve">118-CR0805-FX-1583ELFCT-ND</t>
   </si>
   <si>
-    <t xml:space="preserve">422k Thick Film resistor CRCW0805422KFKEA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/vishay-dale/CRCW0805422KFKEA/1175961 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">541-422KCCT-ND</t>
-  </si>
-  <si>
     <t xml:space="preserve">10k Thick film Resistor RMCF0805FT10K0</t>
   </si>
   <si>
@@ -346,6 +292,42 @@
     <t xml:space="preserve">1712-RLC73PD2BR169FTDCT-ND</t>
   </si>
   <si>
+    <t xml:space="preserve">82k Thick Film resistor CRCW080582K0FKEA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/vishay-dale/CRCW080582K0FKEA/1175855 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">541-82.0KCCT-ND</t>
+  </si>
+  <si>
+    <t xml:space="preserve">100k Thick Film resistor CRCW0805100KFKEA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/vishay-dale/CRCW0805100KFKEA/1175865 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">541-100KCCT-ND</t>
+  </si>
+  <si>
+    <t xml:space="preserve">180 Thick Film resistor RC0805JR-07180RL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/yageo/RC0805JR-07180RL/728263 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">311-180ARCT-ND</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.7k Thick Film Resistor CRG0805F2K7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/te-connectivity-passive-product/CRG0805F2K7/2380883 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">A126359CT-ND</t>
+  </si>
+  <si>
     <t xml:space="preserve">10K LINEAR Potentiometer PDB181-B225K-103B</t>
   </si>
   <si>
@@ -353,234 +335,6 @@
   </si>
   <si>
     <t xml:space="preserve">PDB181-B225K-103B</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">82k </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Thick Film resistor</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> CRCW080582K0FKEA</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/vishay-dale/CRCW080582K0FKEA/1175855</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">541-82.0KCCT-ND</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">100k </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Thick Film resistor CRCW0805100KFKEA</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/vishay-dale/CRCW0805100KFKEA/1175865</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">541-100KCCT-ND</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">180 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Thick Film resistor</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> RC0805JR-07180RL</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/yageo/RC0805JR-07180RL/728263</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">311-180ARCT-ND</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.7k Thick Film Resistor CRG0805F2K7</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/te-connectivity-passive-product/CRG0805F2K7/2380883</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">A126359CT-ND</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Orange LED 2mA XZCM2MOK54WA-1VF</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/sunled/XZCM2MOK54WA-1VF/15761908</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">1497-XZCM2MOK54WA-1VFCT-ND</t>
-  </si>
-  <si>
-    <t xml:space="preserve">White LED 5mA LW Q98G.01-R2T1-3K6L-1-5-R18</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/ams-osram-ag/LW-Q98G-01-R2T1-3K6L-1-5-R18/21556497</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">475-LWQ98G.01-R2T1-3K6L-1CT-ND</t>
   </si>
   <si>
     <t xml:space="preserve">add female connectors for raspberry pi pico</t>
@@ -597,7 +351,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="[$$-1409]#,##0.00;[RED]\-[$$-1409]#,##0.00"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="9">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -647,18 +401,6 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="12"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
       <b val="true"/>
       <u val="single"/>
       <sz val="12"/>
@@ -715,7 +457,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="23">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -768,11 +510,11 @@
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -789,50 +531,18 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1030,7 +740,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="102.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="34.4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="10.06"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="10.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="10.43"/>
   </cols>
   <sheetData>
     <row r="2" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1106,14 +816,14 @@
         <v>14</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F5" s="7" t="n">
         <v>14.04</v>
       </c>
       <c r="G5" s="8" t="n">
         <f aca="false">E5*F5</f>
-        <v>14.04</v>
+        <v>0</v>
       </c>
       <c r="H5" s="9" t="s">
         <v>15</v>
@@ -1130,14 +840,14 @@
         <v>18</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F6" s="7" t="n">
         <v>14.04</v>
       </c>
       <c r="G6" s="8" t="n">
         <f aca="false">E6*F6</f>
-        <v>14.04</v>
+        <v>0</v>
       </c>
       <c r="H6" s="9" t="s">
         <v>15</v>
@@ -1248,58 +958,52 @@
         <v>0.49</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="10"/>
-      <c r="C12" s="10"/>
-      <c r="D12" s="10"/>
-      <c r="E12" s="10"/>
-      <c r="F12" s="13"/>
+    <row r="12" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B12" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="D12" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="E12" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="12" t="n">
+        <v>0.84</v>
+      </c>
       <c r="G12" s="8" t="n">
         <f aca="false">E12*F12</f>
-        <v>0</v>
+        <v>0.84</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="10" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="E13" s="6" t="n">
         <v>1</v>
       </c>
       <c r="F13" s="12" t="n">
-        <v>0.18</v>
+        <v>0.31</v>
       </c>
       <c r="G13" s="8" t="n">
         <f aca="false">E13*F13</f>
-        <v>0.18</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="10" t="s">
-        <v>37</v>
-      </c>
-      <c r="C14" s="11" t="s">
-        <v>38</v>
-      </c>
-      <c r="D14" s="10" t="s">
-        <v>39</v>
-      </c>
-      <c r="E14" s="6"/>
-      <c r="F14" s="12" t="n">
-        <v>0.18</v>
-      </c>
-      <c r="G14" s="8" t="n">
-        <f aca="false">E14*F14</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>0.31</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F14" s="13"/>
+    </row>
+    <row r="15" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B15" s="10" t="s">
         <v>40</v>
       </c>
@@ -1309,247 +1013,240 @@
       <c r="D15" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="E15" s="6"/>
+      <c r="E15" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="F15" s="12" t="n">
-        <v>0.86</v>
+        <v>2.46</v>
       </c>
       <c r="G15" s="8" t="n">
         <f aca="false">E15*F15</f>
-        <v>0</v>
+        <v>2.46</v>
       </c>
       <c r="I15" s="14" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="10"/>
-      <c r="C16" s="11"/>
-      <c r="D16" s="10"/>
-      <c r="E16" s="6"/>
-      <c r="F16" s="12"/>
+      <c r="B16" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="C16" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="D16" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="E16" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" s="12" t="n">
+        <v>1.15</v>
+      </c>
       <c r="G16" s="8" t="n">
         <f aca="false">E16*F16</f>
-        <v>0</v>
+        <v>1.15</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="10" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="C17" s="11" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D17" s="10" t="s">
-        <v>46</v>
-      </c>
-      <c r="E17" s="6"/>
+        <v>49</v>
+      </c>
+      <c r="E17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="F17" s="12" t="n">
-        <v>0.18</v>
+        <v>0.29</v>
       </c>
       <c r="G17" s="8" t="n">
         <f aca="false">E17*F17</f>
-        <v>0</v>
+        <v>0.29</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="10" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="D18" s="10" t="s">
-        <v>49</v>
-      </c>
-      <c r="E18" s="6"/>
+        <v>52</v>
+      </c>
+      <c r="E18" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="F18" s="12" t="n">
         <v>0.18</v>
       </c>
       <c r="G18" s="8" t="n">
         <f aca="false">E18*F18</f>
-        <v>0</v>
+        <v>0.36</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="15" t="s">
-        <v>50</v>
-      </c>
-      <c r="C19" s="16" t="s">
-        <v>51</v>
-      </c>
-      <c r="D19" s="15" t="s">
-        <v>52</v>
-      </c>
-      <c r="E19" s="17" t="n">
-        <v>2</v>
-      </c>
-      <c r="F19" s="18" t="n">
-        <v>0.57</v>
-      </c>
-      <c r="G19" s="19" t="n">
+      <c r="B19" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="C19" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="D19" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="E19" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" s="12" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="G19" s="8" t="n">
         <f aca="false">E19*F19</f>
-        <v>1.14</v>
-      </c>
-      <c r="H19" s="20"/>
-      <c r="I19" s="20" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="10" t="s">
-        <v>54</v>
-      </c>
-      <c r="C20" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="D20" s="10" t="s">
-        <v>56</v>
-      </c>
-      <c r="E20" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F20" s="12" t="n">
-        <v>1.43</v>
-      </c>
-      <c r="G20" s="8" t="n">
-        <f aca="false">E20*F20</f>
-        <v>1.43</v>
-      </c>
+        <v>0.31</v>
+      </c>
+      <c r="I19" s="0"/>
+    </row>
+    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F20" s="13"/>
     </row>
     <row r="21" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="C21" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="C21" s="11" t="s">
+      <c r="D21" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="D21" s="10" t="s">
-        <v>59</v>
-      </c>
       <c r="E21" s="6" t="n">
         <v>1</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>2.46</v>
+        <v>0.18</v>
       </c>
       <c r="G21" s="8" t="n">
         <f aca="false">E21*F21</f>
-        <v>2.46</v>
+        <v>0.18</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="C22" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="C22" s="11" t="s">
+      <c r="D22" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="D22" s="10" t="s">
-        <v>62</v>
-      </c>
       <c r="E22" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>0.31</v>
+        <v>0.18</v>
       </c>
       <c r="G22" s="8" t="n">
         <f aca="false">E22*F22</f>
-        <v>0.31</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>0.36</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="C23" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="C23" s="21" t="s">
+      <c r="D23" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="D23" s="10" t="s">
-        <v>65</v>
-      </c>
       <c r="E23" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="F23" s="22" t="n">
-        <v>1.15</v>
+      <c r="F23" s="12" t="n">
+        <v>0.86</v>
       </c>
       <c r="G23" s="8" t="n">
         <f aca="false">E23*F23</f>
-        <v>1.15</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="23" t="s">
+        <v>0.86</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B24" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="C24" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="C24" s="24" t="s">
+      <c r="D24" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="D24" s="23" t="s">
-        <v>68</v>
-      </c>
-      <c r="E24" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="F24" s="22" t="n">
-        <v>0.29</v>
+      <c r="E24" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F24" s="12" t="n">
+        <v>0.18</v>
       </c>
       <c r="G24" s="8" t="n">
         <f aca="false">E24*F24</f>
-        <v>0.29</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="23" t="s">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B25" s="15" t="s">
+        <v>68</v>
+      </c>
+      <c r="C25" s="16" t="s">
         <v>69</v>
       </c>
-      <c r="C25" s="24" t="s">
+      <c r="D25" s="15" t="s">
         <v>70</v>
       </c>
-      <c r="D25" s="23" t="s">
+      <c r="E25" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="F25" s="18" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="G25" s="19" t="n">
+        <f aca="false">E25*F25</f>
+        <v>0.57</v>
+      </c>
+      <c r="H25" s="20"/>
+      <c r="I25" s="20" t="s">
         <v>71</v>
       </c>
-      <c r="E25" s="25" t="n">
-        <v>2</v>
-      </c>
-      <c r="F25" s="22" t="n">
-        <v>0.18</v>
-      </c>
-      <c r="G25" s="8" t="n">
-        <f aca="false">E25*F25</f>
-        <v>0.36</v>
-      </c>
     </row>
     <row r="26" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="0"/>
-      <c r="C26" s="0"/>
-      <c r="D26" s="0"/>
-      <c r="E26" s="0"/>
-      <c r="F26" s="26"/>
+      <c r="B26" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="C26" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="D26" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="E26" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F26" s="12" t="n">
+        <v>1.43</v>
+      </c>
       <c r="G26" s="8" t="n">
         <f aca="false">E26*F26</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="10" t="s">
-        <v>72</v>
-      </c>
-      <c r="C27" s="11" t="s">
-        <v>73</v>
-      </c>
-      <c r="D27" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="E27" s="6"/>
-      <c r="F27" s="12" t="n">
-        <v>0.18</v>
-      </c>
-      <c r="G27" s="8" t="n">
-        <f aca="false">E27*F27</f>
-        <v>0</v>
-      </c>
+        <v>1.43</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F27" s="13"/>
     </row>
     <row r="28" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="10" t="s">
@@ -1561,13 +1258,15 @@
       <c r="D28" s="10" t="s">
         <v>77</v>
       </c>
-      <c r="E28" s="6"/>
+      <c r="E28" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="F28" s="12" t="n">
         <v>0.18</v>
       </c>
       <c r="G28" s="8" t="n">
         <f aca="false">E28*F28</f>
-        <v>0</v>
+        <v>0.18</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1580,13 +1279,15 @@
       <c r="D29" s="10" t="s">
         <v>80</v>
       </c>
-      <c r="E29" s="6"/>
+      <c r="E29" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="F29" s="12" t="n">
         <v>0.18</v>
       </c>
       <c r="G29" s="8" t="n">
         <f aca="false">E29*F29</f>
-        <v>0</v>
+        <v>0.18</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1599,13 +1300,15 @@
       <c r="D30" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="E30" s="6"/>
+      <c r="E30" s="6" t="n">
+        <v>4</v>
+      </c>
       <c r="F30" s="12" t="n">
         <v>0.18</v>
       </c>
       <c r="G30" s="8" t="n">
         <f aca="false">E30*F30</f>
-        <v>0</v>
+        <v>0.72</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1618,13 +1321,15 @@
       <c r="D31" s="10" t="s">
         <v>86</v>
       </c>
-      <c r="E31" s="6"/>
+      <c r="E31" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="F31" s="12" t="n">
         <v>0.18</v>
       </c>
       <c r="G31" s="8" t="n">
         <f aca="false">E31*F31</f>
-        <v>0</v>
+        <v>0.36</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1637,16 +1342,18 @@
       <c r="D32" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="E32" s="6"/>
+      <c r="E32" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="F32" s="12" t="n">
         <v>0.6</v>
       </c>
       <c r="G32" s="8" t="n">
         <f aca="false">E32*F32</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="10" t="s">
         <v>90</v>
       </c>
@@ -1656,202 +1363,137 @@
       <c r="D33" s="10" t="s">
         <v>92</v>
       </c>
-      <c r="E33" s="6"/>
+      <c r="E33" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="F33" s="12" t="n">
-        <v>2.36</v>
+        <v>0.18</v>
       </c>
       <c r="G33" s="8" t="n">
         <f aca="false">E33*F33</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B34" s="10"/>
-      <c r="C34" s="10"/>
-      <c r="D34" s="10"/>
-      <c r="E34" s="6"/>
-      <c r="F34" s="12"/>
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B34" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="C34" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="D34" s="10" t="s">
+        <v>95</v>
+      </c>
+      <c r="E34" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F34" s="12" t="n">
+        <v>0.18</v>
+      </c>
       <c r="G34" s="8" t="n">
         <f aca="false">E34*F34</f>
-        <v>0</v>
+        <v>0.18</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B35" s="27" t="s">
-        <v>93</v>
-      </c>
-      <c r="C35" s="21" t="s">
-        <v>94</v>
+      <c r="B35" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="C35" s="11" t="s">
+        <v>97</v>
       </c>
       <c r="D35" s="10" t="s">
-        <v>95</v>
-      </c>
-      <c r="E35" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="F35" s="22" t="n">
+        <v>98</v>
+      </c>
+      <c r="E35" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="F35" s="12" t="n">
         <v>0.18</v>
       </c>
       <c r="G35" s="8" t="n">
         <f aca="false">E35*F35</f>
+        <v>0.72</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B36" s="10" t="s">
+        <v>99</v>
+      </c>
+      <c r="C36" s="11" t="s">
+        <v>100</v>
+      </c>
+      <c r="D36" s="10" t="s">
+        <v>101</v>
+      </c>
+      <c r="E36" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F36" s="12" t="n">
         <v>0.18</v>
       </c>
-    </row>
-    <row r="36" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B36" s="27"/>
-      <c r="C36" s="10"/>
-      <c r="D36" s="10"/>
-      <c r="E36" s="6"/>
-      <c r="F36" s="22"/>
       <c r="G36" s="8" t="n">
         <f aca="false">E36*F36</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B37" s="10"/>
-      <c r="C37" s="10"/>
-      <c r="D37" s="10"/>
-      <c r="E37" s="6"/>
-      <c r="F37" s="22"/>
+        <v>0.36</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B37" s="10" t="s">
+        <v>102</v>
+      </c>
+      <c r="C37" s="11" t="s">
+        <v>103</v>
+      </c>
+      <c r="D37" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="E37" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F37" s="12" t="n">
+        <v>2.36</v>
+      </c>
       <c r="G37" s="8" t="n">
         <f aca="false">E37*F37</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B38" s="27"/>
-      <c r="C38" s="10"/>
-      <c r="D38" s="10"/>
-      <c r="E38" s="6"/>
-      <c r="F38" s="22"/>
-      <c r="G38" s="8" t="n">
-        <f aca="false">E38*F38</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B39" s="10"/>
-      <c r="C39" s="10"/>
-      <c r="D39" s="10"/>
-      <c r="E39" s="6"/>
-      <c r="F39" s="12"/>
-      <c r="G39" s="8" t="n">
-        <f aca="false">E39*F39</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B40" s="27" t="s">
-        <v>96</v>
-      </c>
-      <c r="C40" s="21" t="s">
-        <v>97</v>
-      </c>
-      <c r="D40" s="10" t="s">
-        <v>98</v>
-      </c>
-      <c r="E40" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F40" s="12" t="n">
-        <v>0.18</v>
-      </c>
-      <c r="G40" s="8" t="n">
-        <f aca="false">E40*F40</f>
-        <v>0.18</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B41" s="10" t="s">
-        <v>99</v>
-      </c>
-      <c r="C41" s="21" t="s">
-        <v>100</v>
-      </c>
-      <c r="D41" s="10" t="s">
-        <v>101</v>
-      </c>
-      <c r="E41" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="F41" s="12" t="n">
-        <v>0.18</v>
-      </c>
-      <c r="G41" s="8" t="n">
-        <f aca="false">E41*F41</f>
-        <v>0.72</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B42" s="10" t="s">
-        <v>102</v>
-      </c>
-      <c r="C42" s="21" t="s">
-        <v>103</v>
-      </c>
-      <c r="D42" s="10" t="s">
-        <v>104</v>
-      </c>
-      <c r="E42" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F42" s="28" t="n">
-        <v>0.18</v>
-      </c>
-      <c r="G42" s="8" t="n">
-        <f aca="false">E42*F42</f>
-        <v>0.36</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B43" s="10" t="s">
-        <v>105</v>
-      </c>
-      <c r="C43" s="21" t="s">
-        <v>106</v>
-      </c>
-      <c r="D43" s="10" t="s">
-        <v>107</v>
-      </c>
-      <c r="E43" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F43" s="28" t="n">
-        <v>0.84</v>
-      </c>
-      <c r="G43" s="8" t="n">
-        <f aca="false">E43*F43</f>
-        <v>0.84</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B44" s="10" t="s">
-        <v>108</v>
-      </c>
-      <c r="C44" s="21" t="s">
-        <v>109</v>
-      </c>
-      <c r="D44" s="10" t="s">
-        <v>110</v>
-      </c>
-      <c r="E44" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F44" s="28" t="n">
-        <v>0.31</v>
-      </c>
-      <c r="G44" s="8" t="n">
-        <f aca="false">E44*F44</f>
-        <v>0.31</v>
-      </c>
+        <v>2.36</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B38" s="0"/>
+      <c r="C38" s="0"/>
+      <c r="D38" s="0"/>
+      <c r="E38" s="0"/>
+    </row>
+    <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B39" s="0"/>
+      <c r="C39" s="0"/>
+      <c r="D39" s="0"/>
+      <c r="E39" s="0"/>
+    </row>
+    <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B40" s="0"/>
+      <c r="C40" s="0"/>
+      <c r="D40" s="0"/>
+      <c r="E40" s="0"/>
+    </row>
+    <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F41" s="13"/>
+    </row>
+    <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F42" s="13"/>
+    </row>
+    <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F43" s="13"/>
+    </row>
+    <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F44" s="13"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B45" s="10"/>
       <c r="C45" s="10"/>
       <c r="D45" s="10"/>
       <c r="E45" s="6"/>
-      <c r="F45" s="28"/>
+      <c r="F45" s="12"/>
       <c r="G45" s="8" t="n">
         <f aca="false">E45*F45</f>
         <v>0</v>
@@ -1859,12 +1501,12 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B46" s="10"/>
-      <c r="C46" s="29" t="s">
-        <v>111</v>
+      <c r="C46" s="21" t="s">
+        <v>105</v>
       </c>
       <c r="D46" s="10"/>
       <c r="E46" s="6"/>
-      <c r="F46" s="28"/>
+      <c r="F46" s="12"/>
       <c r="G46" s="8" t="n">
         <f aca="false">E46*F46</f>
         <v>0</v>
@@ -1875,19 +1517,19 @@
       <c r="C47" s="10"/>
       <c r="D47" s="10"/>
       <c r="E47" s="6"/>
+      <c r="F47" s="13"/>
       <c r="G47" s="8" t="n">
         <f aca="false">E47*F47</f>
         <v>0</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E48" s="0"/>
       <c r="F48" s="6" t="s">
-        <v>112</v>
-      </c>
-      <c r="G48" s="30" t="n">
+        <v>106</v>
+      </c>
+      <c r="G48" s="22" t="n">
         <f aca="false">SUM(G3:G46)</f>
-        <v>46.96</v>
+        <v>24.11</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2040,31 +1682,29 @@
     <hyperlink ref="C9" r:id="rId7" display="https://www.digikey.co.nz/en/products/detail/w%C3%BCrth-elektronik/691137710004/6644053 "/>
     <hyperlink ref="C10" r:id="rId8" display="https://www.digikey.co.nz/en/products/detail/kingbright/WP813GD/3084264 "/>
     <hyperlink ref="C11" r:id="rId9" display="https://www.digikey.co.nz/en/products/detail/te-connectivity-alcoswitch-switches/1-1825027-1/1632544 "/>
-    <hyperlink ref="C13" r:id="rId10" display="https://www.digikey.co.nz/en/products/detail/w%C3%BCrth-elektronik/860010672004/5726903"/>
-    <hyperlink ref="C14" r:id="rId11" display="https://www.digikey.co.nz/en/products/detail/samsung-electro-mechanics/CL21B104KBCNNNC/3886661 "/>
-    <hyperlink ref="C15" r:id="rId12" display="https://www.digikey.co.nz/en/products/detail/tdk/C2012X5R1V106K125AC/3951654 "/>
-    <hyperlink ref="C17" r:id="rId13" display="https://www.digikey.co.nz/en/products/detail/murata-electronics/GCM1885C2A470JA16J/2591757 "/>
-    <hyperlink ref="C18" r:id="rId14" display="https://www.digikey.co.nz/en/products/detail/kyocera-avx/KGM15ACG2A120JM/1598332 "/>
-    <hyperlink ref="C19" r:id="rId15" display="https://www.digikey.co.nz/en/products/detail/taiyo-yuden/JMK212BBJ476MG-T/4970731 "/>
-    <hyperlink ref="C20" r:id="rId16" display="https://www.digikey.co.nz/en/products/detail/tdk/SLF7045T-6R8M1R7-PF/755381 "/>
-    <hyperlink ref="C21" r:id="rId17" display="https://www.digikey.co.nz/en/products/detail/onsemi/FQD8P10TM/1054070 "/>
-    <hyperlink ref="C22" r:id="rId18" display="https://www.digikey.co.nz/en/products/detail/onsemi/MM3Z24VT1G/661665 "/>
-    <hyperlink ref="C23" r:id="rId19" display="https://www.digikey.co.nz/en/products/detail/diodes-incorporated/DMP3056L-7/5126843"/>
-    <hyperlink ref="C24" r:id="rId20" display="https://www.digikey.co.nz/en/products/detail/nexperia-usa-inc/NX138BKR/5981270"/>
-    <hyperlink ref="C25" r:id="rId21" display="https://www.digikey.co.nz/en/products/detail/shenzhen-slkormicro-semicon-co-ltd/SLMT320V3CN/29782446"/>
-    <hyperlink ref="C27" r:id="rId22" display="https://www.digikey.co.nz/en/products/detail/bourns-inc/CR0805-FX-3012ELF/3784840 "/>
-    <hyperlink ref="C28" r:id="rId23" display="https://www.digikey.co.nz/en/products/detail/bourns-inc/CR0805-FX-1583ELF/3784668 "/>
-    <hyperlink ref="C29" r:id="rId24" display="https://www.digikey.co.nz/en/products/detail/vishay-dale/CRCW0805422KFKEA/1175961 "/>
+    <hyperlink ref="C12" r:id="rId10" display="https://www.digikey.co.nz/en/products/detail/sunled/XZCM2MOK54WA-1VF/15761908 "/>
+    <hyperlink ref="C13" r:id="rId11" display="https://www.digikey.co.nz/en/products/detail/ams-osram-ag/LW-Q98G-01-R2T1-3K6L-1-5-R18/21556497 "/>
+    <hyperlink ref="C15" r:id="rId12" display="https://www.digikey.co.nz/en/products/detail/onsemi/FQD8P10TM/1054070 "/>
+    <hyperlink ref="C16" r:id="rId13" display="https://www.digikey.co.nz/en/products/detail/diodes-incorporated/DMP3056L-7/5126843 "/>
+    <hyperlink ref="C17" r:id="rId14" display="https://www.digikey.co.nz/en/products/detail/nexperia-usa-inc/NX138BKR/5981270 "/>
+    <hyperlink ref="C18" r:id="rId15" display="https://www.digikey.co.nz/en/products/detail/shenzhen-slkormicro-semicon-co-ltd/SLMT320V3CN/29782446 "/>
+    <hyperlink ref="C19" r:id="rId16" display="https://www.digikey.co.nz/en/products/detail/onsemi/MM3Z24VT1G/661665 "/>
+    <hyperlink ref="C21" r:id="rId17" display="https://www.digikey.co.nz/en/products/detail/w%C3%BCrth-elektronik/860010672004/5726903"/>
+    <hyperlink ref="C22" r:id="rId18" display="https://www.digikey.co.nz/en/products/detail/samsung-electro-mechanics/CL21B104KBCNNNC/3886661 "/>
+    <hyperlink ref="C23" r:id="rId19" display="https://www.digikey.co.nz/en/products/detail/tdk/C2012X5R1V106K125AC/3951654 "/>
+    <hyperlink ref="C24" r:id="rId20" display="https://www.digikey.co.nz/en/products/detail/murata-electronics/GCM1885C2A470JA16J/2591757 "/>
+    <hyperlink ref="C25" r:id="rId21" display="https://www.digikey.co.nz/en/products/detail/taiyo-yuden/JMK212BBJ476MG-T/4970731 "/>
+    <hyperlink ref="C26" r:id="rId22" display="https://www.digikey.co.nz/en/products/detail/tdk/SLF7045T-6R8M1R7-PF/755381 "/>
+    <hyperlink ref="C28" r:id="rId23" display="https://www.digikey.co.nz/en/products/detail/bourns-inc/CR0805-FX-3012ELF/3784840 "/>
+    <hyperlink ref="C29" r:id="rId24" display="https://www.digikey.co.nz/en/products/detail/bourns-inc/CR0805-FX-1583ELF/3784668 "/>
     <hyperlink ref="C30" r:id="rId25" display="https://www.digikey.co.nz/en/products/detail/stackpole-electronics-inc/RMCF0805FT10K0/1760676 "/>
     <hyperlink ref="C31" r:id="rId26" display="https://www.digikey.co.nz/en/products/detail/stackpole-electronics-inc/RNCP0805FTD1K00/2240229 "/>
     <hyperlink ref="C32" r:id="rId27" display="https://www.digikey.co.nz/en/products/detail/te-connectivity-passive-product/RLC73PD2BR169FTD/19238107 "/>
-    <hyperlink ref="C33" r:id="rId28" display="https://www.digikey.co.nz/en/products/detail/bourns-inc/PDB181-B225K-103B/6153329 "/>
-    <hyperlink ref="C35" r:id="rId29" display="https://www.digikey.co.nz/en/products/detail/vishay-dale/CRCW080582K0FKEA/1175855"/>
-    <hyperlink ref="C40" r:id="rId30" display="https://www.digikey.co.nz/en/products/detail/vishay-dale/CRCW0805100KFKEA/1175865"/>
-    <hyperlink ref="C41" r:id="rId31" display="https://www.digikey.co.nz/en/products/detail/yageo/RC0805JR-07180RL/728263"/>
-    <hyperlink ref="C42" r:id="rId32" display="https://www.digikey.co.nz/en/products/detail/te-connectivity-passive-product/CRG0805F2K7/2380883"/>
-    <hyperlink ref="C43" r:id="rId33" display="https://www.digikey.co.nz/en/products/detail/sunled/XZCM2MOK54WA-1VF/15761908"/>
-    <hyperlink ref="C44" r:id="rId34" display="https://www.digikey.co.nz/en/products/detail/ams-osram-ag/LW-Q98G-01-R2T1-3K6L-1-5-R18/21556497"/>
+    <hyperlink ref="C33" r:id="rId28" display="https://www.digikey.co.nz/en/products/detail/vishay-dale/CRCW080582K0FKEA/1175855 "/>
+    <hyperlink ref="C34" r:id="rId29" display="https://www.digikey.co.nz/en/products/detail/vishay-dale/CRCW0805100KFKEA/1175865 "/>
+    <hyperlink ref="C35" r:id="rId30" display="https://www.digikey.co.nz/en/products/detail/yageo/RC0805JR-07180RL/728263 "/>
+    <hyperlink ref="C36" r:id="rId31" display="https://www.digikey.co.nz/en/products/detail/te-connectivity-passive-product/CRG0805F2K7/2380883 "/>
+    <hyperlink ref="C37" r:id="rId32" display="https://www.digikey.co.nz/en/products/detail/bourns-inc/PDB181-B225K-103B/6153329 "/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>

<commit_message>
Finished final schematic and PCB revisions
</commit_message>
<xml_diff>
--- a/Schematics & PCB/parts_order.xlsx
+++ b/Schematics & PCB/parts_order.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="111">
   <si>
     <t xml:space="preserve">Component</t>
   </si>
@@ -142,6 +142,33 @@
     <t xml:space="preserve">475-LWQ98G.01-R2T1-3K6L-1CT-ND</t>
   </si>
   <si>
+    <t xml:space="preserve">20p Female Connector 61302011821</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/w%C3%BCrth-elektronik/61302011821/16608603</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">732-61302011821-ND</t>
+  </si>
+  <si>
     <t xml:space="preserve">PMOS 100V 6.6A FQD8P10TM</t>
   </si>
   <si>
@@ -208,6 +235,9 @@
     <t xml:space="preserve">1276-1003-1-ND</t>
   </si>
   <si>
+    <t xml:space="preserve">low esr</t>
+  </si>
+  <si>
     <t xml:space="preserve">10uF Ceramic Capacitor C2012X5R1V106K125AC</t>
   </si>
   <si>
@@ -235,7 +265,7 @@
     <t xml:space="preserve">587-4280-1-ND</t>
   </si>
   <si>
-    <t xml:space="preserve">might need to find high esr</t>
+    <t xml:space="preserve">if you can*</t>
   </si>
   <si>
     <t xml:space="preserve">6.8uH Shielded Inductor SLF7045T-6R8M1R7-PF</t>
@@ -351,7 +381,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="[$$-1409]#,##0.00;[RED]\-[$$-1409]#,##0.00"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="11">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -394,11 +424,23 @@
       <charset val="1"/>
     </font>
     <font>
+      <sz val="12"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <b val="true"/>
       <sz val="16"/>
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b val="true"/>
@@ -409,12 +451,18 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFAFD095"/>
+        <bgColor rgb="FF99CCFF"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -457,7 +505,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="38">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -474,6 +522,26 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -510,39 +578,79 @@
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -575,7 +683,7 @@
       <rgbColor rgb="FF808000"/>
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FFC0C0C0"/>
+      <rgbColor rgb="FFAFD095"/>
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
@@ -733,7 +841,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B2:I66"/>
+  <dimension ref="B2:J66"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="48.67"/>
@@ -806,151 +914,151 @@
       </c>
     </row>
     <row r="5" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="E5" s="6" t="n">
+      <c r="E5" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="F5" s="7" t="n">
+      <c r="F5" s="12" t="n">
         <v>14.04</v>
       </c>
-      <c r="G5" s="8" t="n">
+      <c r="G5" s="13" t="n">
         <f aca="false">E5*F5</f>
         <v>0</v>
       </c>
-      <c r="H5" s="9" t="s">
+      <c r="H5" s="14" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="E6" s="6" t="n">
+      <c r="E6" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="F6" s="7" t="n">
+      <c r="F6" s="12" t="n">
         <v>14.04</v>
       </c>
-      <c r="G6" s="8" t="n">
+      <c r="G6" s="13" t="n">
         <f aca="false">E6*F6</f>
         <v>0</v>
       </c>
-      <c r="H6" s="9" t="s">
+      <c r="H6" s="14" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="10" t="s">
+      <c r="B7" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="C7" s="11" t="s">
+      <c r="C7" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="D7" s="10" t="s">
+      <c r="D7" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="E7" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F7" s="12" t="n">
+      <c r="E7" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" s="17" t="n">
         <v>0.62</v>
       </c>
-      <c r="G7" s="8" t="n">
+      <c r="G7" s="13" t="n">
         <f aca="false">E7*F7</f>
         <v>0.62</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="C8" s="11" t="s">
+      <c r="C8" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="D8" s="10" t="s">
+      <c r="D8" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="E8" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F8" s="12" t="n">
+      <c r="E8" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" s="17" t="n">
         <v>0.7</v>
       </c>
-      <c r="G8" s="8" t="n">
+      <c r="G8" s="13" t="n">
         <f aca="false">E8*F8</f>
         <v>0.7</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="10" t="s">
+      <c r="B9" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="C9" s="11" t="s">
+      <c r="C9" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="D9" s="10" t="s">
+      <c r="D9" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="E9" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F9" s="12" t="n">
+      <c r="E9" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" s="17" t="n">
         <v>1.34</v>
       </c>
-      <c r="G9" s="8" t="n">
+      <c r="G9" s="13" t="n">
         <f aca="false">E9*F9</f>
         <v>1.34</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="10" t="s">
+      <c r="B10" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="C10" s="11" t="s">
+      <c r="C10" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="D10" s="10" t="s">
+      <c r="D10" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="E10" s="6" t="n">
+      <c r="E10" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="F10" s="12" t="n">
+      <c r="F10" s="17" t="n">
         <v>0.6</v>
       </c>
-      <c r="G10" s="8" t="n">
+      <c r="G10" s="13" t="n">
         <f aca="false">E10*F10</f>
         <v>1.2</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="10" t="s">
+      <c r="B11" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="C11" s="11" t="s">
+      <c r="C11" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="D11" s="10" t="s">
+      <c r="D11" s="18" t="s">
         <v>33</v>
       </c>
       <c r="E11" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="F11" s="12" t="n">
+      <c r="F11" s="20" t="n">
         <v>0.49</v>
       </c>
       <c r="G11" s="8" t="n">
@@ -959,717 +1067,784 @@
       </c>
     </row>
     <row r="12" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="10" t="s">
+      <c r="B12" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="C12" s="11" t="s">
+      <c r="C12" s="16" t="s">
         <v>35</v>
       </c>
-      <c r="D12" s="10" t="s">
+      <c r="D12" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="E12" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F12" s="12" t="n">
+      <c r="E12" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="17" t="n">
         <v>0.84</v>
       </c>
-      <c r="G12" s="8" t="n">
+      <c r="G12" s="13" t="n">
         <f aca="false">E12*F12</f>
         <v>0.84</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="10" t="s">
+      <c r="B13" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="C13" s="11" t="s">
+      <c r="C13" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="D13" s="10" t="s">
+      <c r="D13" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="E13" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F13" s="12" t="n">
+      <c r="E13" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" s="17" t="n">
         <v>0.31</v>
       </c>
-      <c r="G13" s="8" t="n">
+      <c r="G13" s="13" t="n">
         <f aca="false">E13*F13</f>
         <v>0.31</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F14" s="13"/>
+    <row r="14" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B14" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="C14" s="21" t="s">
+        <v>41</v>
+      </c>
+      <c r="D14" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="E14" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F14" s="20" t="n">
+        <v>1.61</v>
+      </c>
+      <c r="G14" s="22" t="n">
+        <f aca="false">F14*E14</f>
+        <v>3.22</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B15" s="10" t="s">
-        <v>40</v>
-      </c>
-      <c r="C15" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="D15" s="10" t="s">
-        <v>42</v>
-      </c>
-      <c r="E15" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F15" s="12" t="n">
+      <c r="B15" s="23"/>
+      <c r="C15" s="23"/>
+      <c r="D15" s="23"/>
+      <c r="E15" s="23"/>
+      <c r="F15" s="24"/>
+      <c r="G15" s="23"/>
+      <c r="I15" s="0"/>
+    </row>
+    <row r="16" customFormat="false" ht="14.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B16" s="15" t="s">
+        <v>43</v>
+      </c>
+      <c r="C16" s="16" t="s">
+        <v>44</v>
+      </c>
+      <c r="D16" s="15" t="s">
+        <v>45</v>
+      </c>
+      <c r="E16" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" s="17" t="n">
         <v>2.46</v>
       </c>
-      <c r="G15" s="8" t="n">
-        <f aca="false">E15*F15</f>
+      <c r="G16" s="13" t="n">
+        <f aca="false">E16*F16</f>
         <v>2.46</v>
       </c>
-      <c r="I15" s="14" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="C16" s="11" t="s">
-        <v>45</v>
-      </c>
-      <c r="D16" s="10" t="s">
+      <c r="I16" s="25" t="s">
         <v>46</v>
       </c>
-      <c r="E16" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F16" s="12" t="n">
+    </row>
+    <row r="17" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B17" s="15" t="s">
+        <v>47</v>
+      </c>
+      <c r="C17" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="D17" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="E17" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" s="17" t="n">
         <v>1.15</v>
       </c>
-      <c r="G16" s="8" t="n">
-        <f aca="false">E16*F16</f>
+      <c r="G17" s="13" t="n">
+        <f aca="false">E17*F17</f>
         <v>1.15</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="C17" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="D17" s="10" t="s">
-        <v>49</v>
-      </c>
-      <c r="E17" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F17" s="12" t="n">
+    <row r="18" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B18" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="C18" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="D18" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="E18" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" s="17" t="n">
         <v>0.29</v>
       </c>
-      <c r="G17" s="8" t="n">
-        <f aca="false">E17*F17</f>
+      <c r="G18" s="13" t="n">
+        <f aca="false">E18*F18</f>
         <v>0.29</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="10" t="s">
-        <v>50</v>
-      </c>
-      <c r="C18" s="11" t="s">
-        <v>51</v>
-      </c>
-      <c r="D18" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="E18" s="6" t="n">
+    <row r="19" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B19" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="C19" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="D19" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="E19" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="F18" s="12" t="n">
+      <c r="F19" s="17" t="n">
         <v>0.18</v>
       </c>
-      <c r="G18" s="8" t="n">
-        <f aca="false">E18*F18</f>
+      <c r="G19" s="13" t="n">
+        <f aca="false">E19*F19</f>
         <v>0.36</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="10" t="s">
-        <v>53</v>
-      </c>
-      <c r="C19" s="11" t="s">
-        <v>54</v>
-      </c>
-      <c r="D19" s="10" t="s">
-        <v>55</v>
-      </c>
-      <c r="E19" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F19" s="12" t="n">
+    <row r="20" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B20" s="15" t="s">
+        <v>56</v>
+      </c>
+      <c r="C20" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="D20" s="15" t="s">
+        <v>58</v>
+      </c>
+      <c r="E20" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F20" s="17" t="n">
         <v>0.31</v>
       </c>
-      <c r="G19" s="8" t="n">
-        <f aca="false">E19*F19</f>
+      <c r="G20" s="13" t="n">
+        <f aca="false">E20*F20</f>
         <v>0.31</v>
       </c>
-      <c r="I19" s="0"/>
-    </row>
-    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F20" s="13"/>
-    </row>
-    <row r="21" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="10" t="s">
-        <v>56</v>
-      </c>
-      <c r="C21" s="11" t="s">
-        <v>57</v>
-      </c>
-      <c r="D21" s="10" t="s">
-        <v>58</v>
-      </c>
-      <c r="E21" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F21" s="12" t="n">
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B21" s="15"/>
+      <c r="C21" s="15"/>
+      <c r="D21" s="15"/>
+      <c r="E21" s="15"/>
+      <c r="F21" s="17"/>
+      <c r="G21" s="23"/>
+    </row>
+    <row r="22" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B22" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="C22" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="D22" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="E22" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F22" s="17" t="n">
         <v>0.18</v>
       </c>
-      <c r="G21" s="8" t="n">
-        <f aca="false">E21*F21</f>
+      <c r="G22" s="13" t="n">
+        <f aca="false">E22*F22</f>
         <v>0.18</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="C22" s="11" t="s">
-        <v>60</v>
-      </c>
-      <c r="D22" s="10" t="s">
-        <v>61</v>
-      </c>
-      <c r="E22" s="6" t="n">
+    <row r="23" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B23" s="15" t="s">
+        <v>62</v>
+      </c>
+      <c r="C23" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="D23" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="E23" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="F22" s="12" t="n">
+      <c r="F23" s="17" t="n">
         <v>0.18</v>
       </c>
-      <c r="G22" s="8" t="n">
-        <f aca="false">E22*F22</f>
+      <c r="G23" s="13" t="n">
+        <f aca="false">E23*F23</f>
         <v>0.36</v>
       </c>
-    </row>
-    <row r="23" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="10" t="s">
-        <v>62</v>
-      </c>
-      <c r="C23" s="11" t="s">
-        <v>63</v>
-      </c>
-      <c r="D23" s="10" t="s">
-        <v>64</v>
-      </c>
-      <c r="E23" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F23" s="12" t="n">
+      <c r="I23" s="26" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B24" s="15" t="s">
+        <v>66</v>
+      </c>
+      <c r="C24" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="D24" s="15" t="s">
+        <v>68</v>
+      </c>
+      <c r="E24" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F24" s="17" t="n">
         <v>0.86</v>
       </c>
-      <c r="G23" s="8" t="n">
-        <f aca="false">E23*F23</f>
+      <c r="G24" s="13" t="n">
+        <f aca="false">E24*F24</f>
         <v>0.86</v>
       </c>
-    </row>
-    <row r="24" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="10" t="s">
+      <c r="I24" s="1" t="s">
         <v>65</v>
-      </c>
-      <c r="C24" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="D24" s="10" t="s">
-        <v>67</v>
-      </c>
-      <c r="E24" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F24" s="12" t="n">
-        <v>0.18</v>
-      </c>
-      <c r="G24" s="8" t="n">
-        <f aca="false">E24*F24</f>
-        <v>0.18</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="15" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C25" s="16" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D25" s="15" t="s">
-        <v>70</v>
-      </c>
-      <c r="E25" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="F25" s="18" t="n">
+        <v>71</v>
+      </c>
+      <c r="E25" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F25" s="17" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="G25" s="13" t="n">
+        <f aca="false">E25*F25</f>
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B26" s="27" t="s">
+        <v>72</v>
+      </c>
+      <c r="C26" s="28" t="s">
+        <v>73</v>
+      </c>
+      <c r="D26" s="27" t="s">
+        <v>74</v>
+      </c>
+      <c r="E26" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="F26" s="30" t="n">
         <v>0.57</v>
       </c>
-      <c r="G25" s="19" t="n">
-        <f aca="false">E25*F25</f>
+      <c r="G26" s="31" t="n">
+        <f aca="false">E26*F26</f>
         <v>0.57</v>
       </c>
-      <c r="H25" s="20"/>
-      <c r="I25" s="20" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="10" t="s">
-        <v>72</v>
-      </c>
-      <c r="C26" s="11" t="s">
-        <v>73</v>
-      </c>
-      <c r="D26" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="E26" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F26" s="12" t="n">
+      <c r="H26" s="32"/>
+      <c r="I26" s="33" t="s">
+        <v>65</v>
+      </c>
+      <c r="J26" s="34" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B27" s="15" t="s">
+        <v>76</v>
+      </c>
+      <c r="C27" s="16" t="s">
+        <v>77</v>
+      </c>
+      <c r="D27" s="15" t="s">
+        <v>78</v>
+      </c>
+      <c r="E27" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F27" s="17" t="n">
         <v>1.43</v>
       </c>
-      <c r="G26" s="8" t="n">
-        <f aca="false">E26*F26</f>
+      <c r="G27" s="13" t="n">
+        <f aca="false">E27*F27</f>
         <v>1.43</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F27" s="13"/>
-    </row>
-    <row r="28" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B28" s="10" t="s">
-        <v>75</v>
-      </c>
-      <c r="C28" s="11" t="s">
-        <v>76</v>
-      </c>
-      <c r="D28" s="10" t="s">
-        <v>77</v>
-      </c>
-      <c r="E28" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F28" s="12" t="n">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B28" s="15"/>
+      <c r="C28" s="15"/>
+      <c r="D28" s="15"/>
+      <c r="E28" s="15"/>
+      <c r="F28" s="35"/>
+      <c r="G28" s="23"/>
+    </row>
+    <row r="29" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B29" s="15" t="s">
+        <v>79</v>
+      </c>
+      <c r="C29" s="16" t="s">
+        <v>80</v>
+      </c>
+      <c r="D29" s="15" t="s">
+        <v>81</v>
+      </c>
+      <c r="E29" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F29" s="17" t="n">
         <v>0.18</v>
       </c>
-      <c r="G28" s="8" t="n">
-        <f aca="false">E28*F28</f>
-        <v>0.18</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B29" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="C29" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="D29" s="10" t="s">
-        <v>80</v>
-      </c>
-      <c r="E29" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F29" s="12" t="n">
-        <v>0.18</v>
-      </c>
-      <c r="G29" s="8" t="n">
+      <c r="G29" s="13" t="n">
         <f aca="false">E29*F29</f>
         <v>0.18</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B30" s="10" t="s">
-        <v>81</v>
-      </c>
-      <c r="C30" s="11" t="s">
+      <c r="B30" s="15" t="s">
         <v>82</v>
       </c>
-      <c r="D30" s="10" t="s">
+      <c r="C30" s="16" t="s">
         <v>83</v>
       </c>
-      <c r="E30" s="6" t="n">
+      <c r="D30" s="15" t="s">
+        <v>84</v>
+      </c>
+      <c r="E30" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F30" s="17" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="G30" s="13" t="n">
+        <f aca="false">E30*F30</f>
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B31" s="15" t="s">
+        <v>85</v>
+      </c>
+      <c r="C31" s="16" t="s">
+        <v>86</v>
+      </c>
+      <c r="D31" s="15" t="s">
+        <v>87</v>
+      </c>
+      <c r="E31" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="F30" s="12" t="n">
+      <c r="F31" s="17" t="n">
         <v>0.18</v>
       </c>
-      <c r="G30" s="8" t="n">
-        <f aca="false">E30*F30</f>
+      <c r="G31" s="13" t="n">
+        <f aca="false">E31*F31</f>
         <v>0.72</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B31" s="10" t="s">
-        <v>84</v>
-      </c>
-      <c r="C31" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="D31" s="10" t="s">
-        <v>86</v>
-      </c>
-      <c r="E31" s="6" t="n">
+    <row r="32" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B32" s="15" t="s">
+        <v>88</v>
+      </c>
+      <c r="C32" s="16" t="s">
+        <v>89</v>
+      </c>
+      <c r="D32" s="15" t="s">
+        <v>90</v>
+      </c>
+      <c r="E32" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="F31" s="12" t="n">
+      <c r="F32" s="17" t="n">
         <v>0.18</v>
       </c>
-      <c r="G31" s="8" t="n">
-        <f aca="false">E31*F31</f>
+      <c r="G32" s="13" t="n">
+        <f aca="false">E32*F32</f>
         <v>0.36</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B32" s="10" t="s">
-        <v>87</v>
-      </c>
-      <c r="C32" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="D32" s="10" t="s">
-        <v>89</v>
-      </c>
-      <c r="E32" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F32" s="12" t="n">
+    <row r="33" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B33" s="15" t="s">
+        <v>91</v>
+      </c>
+      <c r="C33" s="16" t="s">
+        <v>92</v>
+      </c>
+      <c r="D33" s="15" t="s">
+        <v>93</v>
+      </c>
+      <c r="E33" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F33" s="17" t="n">
         <v>0.6</v>
       </c>
-      <c r="G32" s="8" t="n">
-        <f aca="false">E32*F32</f>
+      <c r="G33" s="13" t="n">
+        <f aca="false">E33*F33</f>
         <v>0.6</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B33" s="10" t="s">
-        <v>90</v>
-      </c>
-      <c r="C33" s="11" t="s">
-        <v>91</v>
-      </c>
-      <c r="D33" s="10" t="s">
-        <v>92</v>
-      </c>
-      <c r="E33" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F33" s="12" t="n">
+    <row r="34" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B34" s="15" t="s">
+        <v>94</v>
+      </c>
+      <c r="C34" s="16" t="s">
+        <v>95</v>
+      </c>
+      <c r="D34" s="15" t="s">
+        <v>96</v>
+      </c>
+      <c r="E34" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F34" s="17" t="n">
         <v>0.18</v>
       </c>
-      <c r="G33" s="8" t="n">
-        <f aca="false">E33*F33</f>
-        <v>0.18</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B34" s="10" t="s">
-        <v>93</v>
-      </c>
-      <c r="C34" s="11" t="s">
-        <v>94</v>
-      </c>
-      <c r="D34" s="10" t="s">
-        <v>95</v>
-      </c>
-      <c r="E34" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F34" s="12" t="n">
-        <v>0.18</v>
-      </c>
-      <c r="G34" s="8" t="n">
+      <c r="G34" s="13" t="n">
         <f aca="false">E34*F34</f>
         <v>0.18</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B35" s="10" t="s">
-        <v>96</v>
-      </c>
-      <c r="C35" s="11" t="s">
+      <c r="B35" s="15" t="s">
         <v>97</v>
       </c>
-      <c r="D35" s="10" t="s">
+      <c r="C35" s="16" t="s">
         <v>98</v>
       </c>
-      <c r="E35" s="6" t="n">
+      <c r="D35" s="15" t="s">
+        <v>99</v>
+      </c>
+      <c r="E35" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F35" s="17" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="G35" s="13" t="n">
+        <f aca="false">E35*F35</f>
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B36" s="15" t="s">
+        <v>100</v>
+      </c>
+      <c r="C36" s="16" t="s">
+        <v>101</v>
+      </c>
+      <c r="D36" s="15" t="s">
+        <v>102</v>
+      </c>
+      <c r="E36" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="F35" s="12" t="n">
+      <c r="F36" s="17" t="n">
         <v>0.18</v>
       </c>
-      <c r="G35" s="8" t="n">
-        <f aca="false">E35*F35</f>
+      <c r="G36" s="13" t="n">
+        <f aca="false">E36*F36</f>
         <v>0.72</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B36" s="10" t="s">
-        <v>99</v>
-      </c>
-      <c r="C36" s="11" t="s">
-        <v>100</v>
-      </c>
-      <c r="D36" s="10" t="s">
-        <v>101</v>
-      </c>
-      <c r="E36" s="6" t="n">
+    <row r="37" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B37" s="15" t="s">
+        <v>103</v>
+      </c>
+      <c r="C37" s="16" t="s">
+        <v>104</v>
+      </c>
+      <c r="D37" s="15" t="s">
+        <v>105</v>
+      </c>
+      <c r="E37" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="F36" s="12" t="n">
+      <c r="F37" s="17" t="n">
         <v>0.18</v>
       </c>
-      <c r="G36" s="8" t="n">
-        <f aca="false">E36*F36</f>
+      <c r="G37" s="13" t="n">
+        <f aca="false">E37*F37</f>
         <v>0.36</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B37" s="10" t="s">
-        <v>102</v>
-      </c>
-      <c r="C37" s="11" t="s">
-        <v>103</v>
-      </c>
-      <c r="D37" s="10" t="s">
-        <v>104</v>
-      </c>
-      <c r="E37" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F37" s="12" t="n">
+    <row r="38" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B38" s="15" t="s">
+        <v>106</v>
+      </c>
+      <c r="C38" s="16" t="s">
+        <v>107</v>
+      </c>
+      <c r="D38" s="15" t="s">
+        <v>108</v>
+      </c>
+      <c r="E38" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F38" s="17" t="n">
         <v>2.36</v>
       </c>
-      <c r="G37" s="8" t="n">
-        <f aca="false">E37*F37</f>
+      <c r="G38" s="13" t="n">
+        <f aca="false">E38*F38</f>
         <v>2.36</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B38" s="0"/>
-      <c r="C38" s="0"/>
-      <c r="D38" s="0"/>
-      <c r="E38" s="0"/>
-    </row>
-    <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B39" s="0"/>
-      <c r="C39" s="0"/>
-      <c r="D39" s="0"/>
-      <c r="E39" s="0"/>
-    </row>
-    <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B40" s="0"/>
-      <c r="C40" s="0"/>
-      <c r="D40" s="0"/>
-      <c r="E40" s="0"/>
-    </row>
-    <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F41" s="13"/>
-    </row>
-    <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F42" s="13"/>
-    </row>
-    <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F43" s="13"/>
-    </row>
-    <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F44" s="13"/>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B39" s="15"/>
+      <c r="C39" s="15"/>
+      <c r="D39" s="15"/>
+      <c r="E39" s="15"/>
+      <c r="F39" s="23"/>
+      <c r="G39" s="23"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B40" s="15"/>
+      <c r="C40" s="15"/>
+      <c r="D40" s="15"/>
+      <c r="E40" s="15"/>
+      <c r="F40" s="23"/>
+      <c r="G40" s="23"/>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B41" s="15"/>
+      <c r="C41" s="15"/>
+      <c r="D41" s="15"/>
+      <c r="E41" s="15"/>
+      <c r="F41" s="35"/>
+      <c r="G41" s="23"/>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B42" s="15"/>
+      <c r="C42" s="15"/>
+      <c r="D42" s="15"/>
+      <c r="E42" s="15"/>
+      <c r="F42" s="35"/>
+      <c r="G42" s="23"/>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B43" s="15"/>
+      <c r="C43" s="15"/>
+      <c r="D43" s="15"/>
+      <c r="E43" s="15"/>
+      <c r="F43" s="35"/>
+      <c r="G43" s="23"/>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B44" s="15"/>
+      <c r="C44" s="15"/>
+      <c r="D44" s="15"/>
+      <c r="E44" s="15"/>
+      <c r="F44" s="35"/>
+      <c r="G44" s="23"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B45" s="10"/>
-      <c r="C45" s="10"/>
-      <c r="D45" s="10"/>
-      <c r="E45" s="6"/>
-      <c r="F45" s="12"/>
-      <c r="G45" s="8" t="n">
+      <c r="B45" s="15"/>
+      <c r="C45" s="15"/>
+      <c r="D45" s="15"/>
+      <c r="E45" s="11"/>
+      <c r="F45" s="17"/>
+      <c r="G45" s="13" t="n">
         <f aca="false">E45*F45</f>
         <v>0</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B46" s="10"/>
-      <c r="C46" s="21" t="s">
-        <v>105</v>
-      </c>
-      <c r="D46" s="10"/>
-      <c r="E46" s="6"/>
-      <c r="F46" s="12"/>
-      <c r="G46" s="8" t="n">
+      <c r="B46" s="15"/>
+      <c r="C46" s="36" t="s">
+        <v>109</v>
+      </c>
+      <c r="D46" s="15"/>
+      <c r="E46" s="11"/>
+      <c r="F46" s="17"/>
+      <c r="G46" s="13" t="n">
         <f aca="false">E46*F46</f>
         <v>0</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B47" s="10"/>
-      <c r="C47" s="10"/>
-      <c r="D47" s="10"/>
-      <c r="E47" s="6"/>
-      <c r="F47" s="13"/>
-      <c r="G47" s="8" t="n">
+      <c r="B47" s="15"/>
+      <c r="C47" s="15"/>
+      <c r="D47" s="15"/>
+      <c r="E47" s="11"/>
+      <c r="F47" s="35"/>
+      <c r="G47" s="13" t="n">
         <f aca="false">E47*F47</f>
         <v>0</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F48" s="6" t="s">
-        <v>106</v>
-      </c>
-      <c r="G48" s="22" t="n">
+      <c r="B48" s="15"/>
+      <c r="C48" s="15"/>
+      <c r="D48" s="15"/>
+      <c r="E48" s="15"/>
+      <c r="F48" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="G48" s="37" t="n">
         <f aca="false">SUM(G3:G46)</f>
-        <v>24.11</v>
+        <v>27.33</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G49" s="10"/>
+      <c r="G49" s="15"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B50" s="10"/>
-      <c r="C50" s="10"/>
-      <c r="D50" s="10"/>
-      <c r="E50" s="10"/>
-      <c r="F50" s="10"/>
-      <c r="G50" s="10"/>
+      <c r="B50" s="15"/>
+      <c r="C50" s="15"/>
+      <c r="D50" s="15"/>
+      <c r="E50" s="15"/>
+      <c r="F50" s="15"/>
+      <c r="G50" s="15"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B51" s="10"/>
-      <c r="C51" s="10"/>
-      <c r="D51" s="10"/>
-      <c r="E51" s="10"/>
-      <c r="F51" s="10"/>
-      <c r="G51" s="10"/>
+      <c r="B51" s="15"/>
+      <c r="C51" s="15"/>
+      <c r="D51" s="15"/>
+      <c r="E51" s="15"/>
+      <c r="F51" s="15"/>
+      <c r="G51" s="15"/>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B52" s="10"/>
-      <c r="C52" s="10"/>
-      <c r="D52" s="10"/>
-      <c r="E52" s="10"/>
-      <c r="F52" s="10"/>
-      <c r="G52" s="10"/>
+      <c r="B52" s="15"/>
+      <c r="C52" s="15"/>
+      <c r="D52" s="15"/>
+      <c r="E52" s="15"/>
+      <c r="F52" s="15"/>
+      <c r="G52" s="15"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B53" s="10"/>
-      <c r="C53" s="10"/>
-      <c r="D53" s="10"/>
-      <c r="E53" s="10"/>
-      <c r="F53" s="10"/>
-      <c r="G53" s="10"/>
+      <c r="B53" s="15"/>
+      <c r="C53" s="15"/>
+      <c r="D53" s="15"/>
+      <c r="E53" s="15"/>
+      <c r="F53" s="15"/>
+      <c r="G53" s="15"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B54" s="10"/>
-      <c r="C54" s="10"/>
-      <c r="D54" s="10"/>
-      <c r="E54" s="10"/>
-      <c r="F54" s="10"/>
-      <c r="G54" s="10"/>
+      <c r="B54" s="15"/>
+      <c r="C54" s="15"/>
+      <c r="D54" s="15"/>
+      <c r="E54" s="15"/>
+      <c r="F54" s="15"/>
+      <c r="G54" s="15"/>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B55" s="10"/>
-      <c r="C55" s="10"/>
-      <c r="D55" s="10"/>
-      <c r="E55" s="10"/>
-      <c r="F55" s="10"/>
-      <c r="G55" s="10"/>
+      <c r="B55" s="15"/>
+      <c r="C55" s="15"/>
+      <c r="D55" s="15"/>
+      <c r="E55" s="15"/>
+      <c r="F55" s="15"/>
+      <c r="G55" s="15"/>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B56" s="10"/>
-      <c r="C56" s="10"/>
-      <c r="D56" s="10"/>
-      <c r="E56" s="10"/>
-      <c r="F56" s="10"/>
-      <c r="G56" s="10"/>
+      <c r="B56" s="15"/>
+      <c r="C56" s="15"/>
+      <c r="D56" s="15"/>
+      <c r="E56" s="15"/>
+      <c r="F56" s="15"/>
+      <c r="G56" s="15"/>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B57" s="10"/>
-      <c r="C57" s="10"/>
-      <c r="D57" s="10"/>
-      <c r="E57" s="10"/>
-      <c r="F57" s="10"/>
-      <c r="G57" s="10"/>
+      <c r="B57" s="15"/>
+      <c r="C57" s="15"/>
+      <c r="D57" s="15"/>
+      <c r="E57" s="15"/>
+      <c r="F57" s="15"/>
+      <c r="G57" s="15"/>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B58" s="10"/>
-      <c r="C58" s="10"/>
-      <c r="D58" s="10"/>
-      <c r="E58" s="10"/>
-      <c r="F58" s="10"/>
-      <c r="G58" s="10"/>
+      <c r="B58" s="15"/>
+      <c r="C58" s="15"/>
+      <c r="D58" s="15"/>
+      <c r="E58" s="15"/>
+      <c r="F58" s="15"/>
+      <c r="G58" s="15"/>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B59" s="10"/>
-      <c r="C59" s="10"/>
-      <c r="D59" s="10"/>
-      <c r="E59" s="10"/>
-      <c r="F59" s="10"/>
-      <c r="G59" s="10"/>
+      <c r="B59" s="15"/>
+      <c r="C59" s="15"/>
+      <c r="D59" s="15"/>
+      <c r="E59" s="15"/>
+      <c r="F59" s="15"/>
+      <c r="G59" s="15"/>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B60" s="10"/>
-      <c r="C60" s="10"/>
-      <c r="D60" s="10"/>
-      <c r="E60" s="10"/>
-      <c r="F60" s="10"/>
-      <c r="G60" s="10"/>
+      <c r="B60" s="15"/>
+      <c r="C60" s="15"/>
+      <c r="D60" s="15"/>
+      <c r="E60" s="15"/>
+      <c r="F60" s="15"/>
+      <c r="G60" s="15"/>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B61" s="10"/>
-      <c r="C61" s="10"/>
-      <c r="D61" s="10"/>
-      <c r="E61" s="10"/>
-      <c r="F61" s="10"/>
-      <c r="G61" s="10"/>
+      <c r="B61" s="15"/>
+      <c r="C61" s="15"/>
+      <c r="D61" s="15"/>
+      <c r="E61" s="15"/>
+      <c r="F61" s="15"/>
+      <c r="G61" s="15"/>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B62" s="10"/>
-      <c r="C62" s="10"/>
-      <c r="D62" s="10"/>
-      <c r="E62" s="10"/>
-      <c r="F62" s="10"/>
-      <c r="G62" s="10"/>
+      <c r="B62" s="15"/>
+      <c r="C62" s="15"/>
+      <c r="D62" s="15"/>
+      <c r="E62" s="15"/>
+      <c r="F62" s="15"/>
+      <c r="G62" s="15"/>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B63" s="10"/>
-      <c r="C63" s="10"/>
-      <c r="D63" s="10"/>
-      <c r="E63" s="10"/>
-      <c r="F63" s="10"/>
-      <c r="G63" s="10"/>
+      <c r="B63" s="15"/>
+      <c r="C63" s="15"/>
+      <c r="D63" s="15"/>
+      <c r="E63" s="15"/>
+      <c r="F63" s="15"/>
+      <c r="G63" s="15"/>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B64" s="10"/>
-      <c r="C64" s="10"/>
-      <c r="D64" s="10"/>
-      <c r="E64" s="10"/>
-      <c r="F64" s="10"/>
-      <c r="G64" s="10"/>
+      <c r="B64" s="15"/>
+      <c r="C64" s="15"/>
+      <c r="D64" s="15"/>
+      <c r="E64" s="15"/>
+      <c r="F64" s="15"/>
+      <c r="G64" s="15"/>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B65" s="10"/>
-      <c r="C65" s="10"/>
-      <c r="D65" s="10"/>
-      <c r="E65" s="10"/>
-      <c r="F65" s="10"/>
-      <c r="G65" s="10"/>
+      <c r="B65" s="15"/>
+      <c r="C65" s="15"/>
+      <c r="D65" s="15"/>
+      <c r="E65" s="15"/>
+      <c r="F65" s="15"/>
+      <c r="G65" s="15"/>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B66" s="10"/>
-      <c r="C66" s="10"/>
-      <c r="D66" s="10"/>
-      <c r="E66" s="10"/>
-      <c r="F66" s="10"/>
-      <c r="G66" s="10"/>
+      <c r="B66" s="15"/>
+      <c r="C66" s="15"/>
+      <c r="D66" s="15"/>
+      <c r="E66" s="15"/>
+      <c r="F66" s="15"/>
+      <c r="G66" s="15"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -1684,27 +1859,28 @@
     <hyperlink ref="C11" r:id="rId9" display="https://www.digikey.co.nz/en/products/detail/te-connectivity-alcoswitch-switches/1-1825027-1/1632544 "/>
     <hyperlink ref="C12" r:id="rId10" display="https://www.digikey.co.nz/en/products/detail/sunled/XZCM2MOK54WA-1VF/15761908 "/>
     <hyperlink ref="C13" r:id="rId11" display="https://www.digikey.co.nz/en/products/detail/ams-osram-ag/LW-Q98G-01-R2T1-3K6L-1-5-R18/21556497 "/>
-    <hyperlink ref="C15" r:id="rId12" display="https://www.digikey.co.nz/en/products/detail/onsemi/FQD8P10TM/1054070 "/>
-    <hyperlink ref="C16" r:id="rId13" display="https://www.digikey.co.nz/en/products/detail/diodes-incorporated/DMP3056L-7/5126843 "/>
-    <hyperlink ref="C17" r:id="rId14" display="https://www.digikey.co.nz/en/products/detail/nexperia-usa-inc/NX138BKR/5981270 "/>
-    <hyperlink ref="C18" r:id="rId15" display="https://www.digikey.co.nz/en/products/detail/shenzhen-slkormicro-semicon-co-ltd/SLMT320V3CN/29782446 "/>
-    <hyperlink ref="C19" r:id="rId16" display="https://www.digikey.co.nz/en/products/detail/onsemi/MM3Z24VT1G/661665 "/>
-    <hyperlink ref="C21" r:id="rId17" display="https://www.digikey.co.nz/en/products/detail/w%C3%BCrth-elektronik/860010672004/5726903"/>
-    <hyperlink ref="C22" r:id="rId18" display="https://www.digikey.co.nz/en/products/detail/samsung-electro-mechanics/CL21B104KBCNNNC/3886661 "/>
-    <hyperlink ref="C23" r:id="rId19" display="https://www.digikey.co.nz/en/products/detail/tdk/C2012X5R1V106K125AC/3951654 "/>
-    <hyperlink ref="C24" r:id="rId20" display="https://www.digikey.co.nz/en/products/detail/murata-electronics/GCM1885C2A470JA16J/2591757 "/>
-    <hyperlink ref="C25" r:id="rId21" display="https://www.digikey.co.nz/en/products/detail/taiyo-yuden/JMK212BBJ476MG-T/4970731 "/>
-    <hyperlink ref="C26" r:id="rId22" display="https://www.digikey.co.nz/en/products/detail/tdk/SLF7045T-6R8M1R7-PF/755381 "/>
-    <hyperlink ref="C28" r:id="rId23" display="https://www.digikey.co.nz/en/products/detail/bourns-inc/CR0805-FX-3012ELF/3784840 "/>
-    <hyperlink ref="C29" r:id="rId24" display="https://www.digikey.co.nz/en/products/detail/bourns-inc/CR0805-FX-1583ELF/3784668 "/>
-    <hyperlink ref="C30" r:id="rId25" display="https://www.digikey.co.nz/en/products/detail/stackpole-electronics-inc/RMCF0805FT10K0/1760676 "/>
-    <hyperlink ref="C31" r:id="rId26" display="https://www.digikey.co.nz/en/products/detail/stackpole-electronics-inc/RNCP0805FTD1K00/2240229 "/>
-    <hyperlink ref="C32" r:id="rId27" display="https://www.digikey.co.nz/en/products/detail/te-connectivity-passive-product/RLC73PD2BR169FTD/19238107 "/>
-    <hyperlink ref="C33" r:id="rId28" display="https://www.digikey.co.nz/en/products/detail/vishay-dale/CRCW080582K0FKEA/1175855 "/>
-    <hyperlink ref="C34" r:id="rId29" display="https://www.digikey.co.nz/en/products/detail/vishay-dale/CRCW0805100KFKEA/1175865 "/>
-    <hyperlink ref="C35" r:id="rId30" display="https://www.digikey.co.nz/en/products/detail/yageo/RC0805JR-07180RL/728263 "/>
-    <hyperlink ref="C36" r:id="rId31" display="https://www.digikey.co.nz/en/products/detail/te-connectivity-passive-product/CRG0805F2K7/2380883 "/>
-    <hyperlink ref="C37" r:id="rId32" display="https://www.digikey.co.nz/en/products/detail/bourns-inc/PDB181-B225K-103B/6153329 "/>
+    <hyperlink ref="C14" r:id="rId12" display="https://www.digikey.co.nz/en/products/detail/w%C3%BCrth-elektronik/61302011821/16608603"/>
+    <hyperlink ref="C16" r:id="rId13" display="https://www.digikey.co.nz/en/products/detail/onsemi/FQD8P10TM/1054070 "/>
+    <hyperlink ref="C17" r:id="rId14" display="https://www.digikey.co.nz/en/products/detail/diodes-incorporated/DMP3056L-7/5126843 "/>
+    <hyperlink ref="C18" r:id="rId15" display="https://www.digikey.co.nz/en/products/detail/nexperia-usa-inc/NX138BKR/5981270 "/>
+    <hyperlink ref="C19" r:id="rId16" display="https://www.digikey.co.nz/en/products/detail/shenzhen-slkormicro-semicon-co-ltd/SLMT320V3CN/29782446 "/>
+    <hyperlink ref="C20" r:id="rId17" display="https://www.digikey.co.nz/en/products/detail/onsemi/MM3Z24VT1G/661665 "/>
+    <hyperlink ref="C22" r:id="rId18" display="https://www.digikey.co.nz/en/products/detail/w%C3%BCrth-elektronik/860010672004/5726903"/>
+    <hyperlink ref="C23" r:id="rId19" display="https://www.digikey.co.nz/en/products/detail/samsung-electro-mechanics/CL21B104KBCNNNC/3886661 "/>
+    <hyperlink ref="C24" r:id="rId20" display="https://www.digikey.co.nz/en/products/detail/tdk/C2012X5R1V106K125AC/3951654 "/>
+    <hyperlink ref="C25" r:id="rId21" display="https://www.digikey.co.nz/en/products/detail/murata-electronics/GCM1885C2A470JA16J/2591757 "/>
+    <hyperlink ref="C26" r:id="rId22" display="https://www.digikey.co.nz/en/products/detail/taiyo-yuden/JMK212BBJ476MG-T/4970731 "/>
+    <hyperlink ref="C27" r:id="rId23" display="https://www.digikey.co.nz/en/products/detail/tdk/SLF7045T-6R8M1R7-PF/755381 "/>
+    <hyperlink ref="C29" r:id="rId24" display="https://www.digikey.co.nz/en/products/detail/bourns-inc/CR0805-FX-3012ELF/3784840 "/>
+    <hyperlink ref="C30" r:id="rId25" display="https://www.digikey.co.nz/en/products/detail/bourns-inc/CR0805-FX-1583ELF/3784668 "/>
+    <hyperlink ref="C31" r:id="rId26" display="https://www.digikey.co.nz/en/products/detail/stackpole-electronics-inc/RMCF0805FT10K0/1760676 "/>
+    <hyperlink ref="C32" r:id="rId27" display="https://www.digikey.co.nz/en/products/detail/stackpole-electronics-inc/RNCP0805FTD1K00/2240229 "/>
+    <hyperlink ref="C33" r:id="rId28" display="https://www.digikey.co.nz/en/products/detail/te-connectivity-passive-product/RLC73PD2BR169FTD/19238107 "/>
+    <hyperlink ref="C34" r:id="rId29" display="https://www.digikey.co.nz/en/products/detail/vishay-dale/CRCW080582K0FKEA/1175855 "/>
+    <hyperlink ref="C35" r:id="rId30" display="https://www.digikey.co.nz/en/products/detail/vishay-dale/CRCW0805100KFKEA/1175865 "/>
+    <hyperlink ref="C36" r:id="rId31" display="https://www.digikey.co.nz/en/products/detail/yageo/RC0805JR-07180RL/728263 "/>
+    <hyperlink ref="C37" r:id="rId32" display="https://www.digikey.co.nz/en/products/detail/te-connectivity-passive-product/CRG0805F2K7/2380883 "/>
+    <hyperlink ref="C38" r:id="rId33" display="https://www.digikey.co.nz/en/products/detail/bourns-inc/PDB181-B225K-103B/6153329 "/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>

<commit_message>
Finished parts order and added DRC and ERC saves
</commit_message>
<xml_diff>
--- a/Schematics & PCB/parts_order.xlsx
+++ b/Schematics & PCB/parts_order.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="107">
   <si>
     <t xml:space="preserve">Component</t>
   </si>
@@ -67,9 +67,6 @@
     <t xml:space="preserve">4654-FCR7350R-ND </t>
   </si>
   <si>
-    <t xml:space="preserve">try to find better cost</t>
-  </si>
-  <si>
     <t xml:space="preserve">Black Banana socket </t>
   </si>
   <si>
@@ -145,25 +142,7 @@
     <t xml:space="preserve">20p Female Connector 61302011821</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/w%C3%BCrth-elektronik/61302011821/16608603</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
+    <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/w%C3%BCrth-elektronik/61302011821/16608603 </t>
   </si>
   <si>
     <t xml:space="preserve">732-61302011821-ND</t>
@@ -178,9 +157,6 @@
     <t xml:space="preserve">FQD8P10TMCT-ND</t>
   </si>
   <si>
-    <t xml:space="preserve">DOUBLE CHECK THE AMOUNTS AND STUFF</t>
-  </si>
-  <si>
     <t xml:space="preserve">PMOS 30V 4.3A DMP3056L-7</t>
   </si>
   <si>
@@ -217,13 +193,13 @@
     <t xml:space="preserve">MM3Z24VT1GOSCT-ND</t>
   </si>
   <si>
-    <t xml:space="preserve">47uF Al Electrolytic Capacitor 860010372004</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/w%C3%BCrth-elektronik/860010672004/5726903</t>
-  </si>
-  <si>
-    <t xml:space="preserve">732-8596-1-ND</t>
+    <t xml:space="preserve">47uF Al Electrolytic Capacitor 860010572005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/w%C3%BCrth-elektronik/860010572005/5726976 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">732-8735-1-ND</t>
   </si>
   <si>
     <t xml:space="preserve">100nF Ceramic Capacitor CL21B104KBCNNNC</t>
@@ -235,13 +211,13 @@
     <t xml:space="preserve">1276-1003-1-ND</t>
   </si>
   <si>
-    <t xml:space="preserve">low esr</t>
+    <t xml:space="preserve">low esr checked</t>
   </si>
   <si>
     <t xml:space="preserve">10uF Ceramic Capacitor C2012X5R1V106K125AC</t>
   </si>
   <si>
-    <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/tdk/C2012X5R1V106K125AC/3951654 </t>
+    <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/tdk/C2012X5R1V106K085AC/3956083 </t>
   </si>
   <si>
     <t xml:space="preserve">445-14418-1-ND</t>
@@ -256,16 +232,13 @@
     <t xml:space="preserve">490-GCM1885C2A470JA16JCT-ND</t>
   </si>
   <si>
-    <t xml:space="preserve">47uF Ceramic Capacitor JMK212BBJ476MG-T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/taiyo-yuden/JMK212BBJ476MG-T/4970731 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">587-4280-1-ND</t>
-  </si>
-  <si>
-    <t xml:space="preserve">if you can*</t>
+    <t xml:space="preserve">47uF Ceramic Capacitor C2012X5R0J476M125AC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.co.nz/en/products/detail/tdk/C2012X5R0J476M125AC/2443465 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">445-5987-1-ND</t>
   </si>
   <si>
     <t xml:space="preserve">6.8uH Shielded Inductor SLF7045T-6R8M1R7-PF</t>
@@ -365,9 +338,6 @@
   </si>
   <si>
     <t xml:space="preserve">PDB181-B225K-103B</t>
-  </si>
-  <si>
-    <t xml:space="preserve">add female connectors for raspberry pi pico</t>
   </si>
   <si>
     <t xml:space="preserve">TOTAL</t>
@@ -381,7 +351,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="[$$-1409]#,##0.00;[RED]\-[$$-1409]#,##0.00"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="9">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -424,23 +394,11 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="12"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="1"/>
-    </font>
-    <font>
       <b val="true"/>
       <sz val="16"/>
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
     <font>
       <b val="true"/>
@@ -451,7 +409,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -462,12 +420,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFAFD095"/>
         <bgColor rgb="FF99CCFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF6F9D4"/>
-        <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -505,7 +457,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="24">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -566,11 +518,23 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -578,84 +542,16 @@
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -687,7 +583,7 @@
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFF6F9D4"/>
+      <rgbColor rgb="FFFFFFCC"/>
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
@@ -848,6 +744,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="102.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="34.4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="10.06"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="14.65"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="10.43"/>
   </cols>
   <sheetData>
@@ -933,19 +830,17 @@
         <f aca="false">E5*F5</f>
         <v>0</v>
       </c>
-      <c r="H5" s="14" t="s">
-        <v>15</v>
-      </c>
+      <c r="H5" s="14"/>
     </row>
     <row r="6" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="D6" s="9" t="s">
         <v>17</v>
-      </c>
-      <c r="D6" s="9" t="s">
-        <v>18</v>
       </c>
       <c r="E6" s="11" t="n">
         <v>0</v>
@@ -957,108 +852,106 @@
         <f aca="false">E6*F6</f>
         <v>0</v>
       </c>
-      <c r="H6" s="14" t="s">
-        <v>15</v>
-      </c>
+      <c r="H6" s="14"/>
     </row>
     <row r="7" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="C7" s="16" t="s">
+      <c r="D7" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="D7" s="15" t="s">
-        <v>21</v>
-      </c>
-      <c r="E7" s="11" t="n">
+      <c r="E7" s="6" t="n">
         <v>1</v>
       </c>
       <c r="F7" s="17" t="n">
         <v>0.62</v>
       </c>
-      <c r="G7" s="13" t="n">
+      <c r="G7" s="8" t="n">
         <f aca="false">E7*F7</f>
         <v>0.62</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="C8" s="16" t="s">
+      <c r="D8" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="D8" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="E8" s="11" t="n">
+      <c r="E8" s="6" t="n">
         <v>1</v>
       </c>
       <c r="F8" s="17" t="n">
         <v>0.7</v>
       </c>
-      <c r="G8" s="13" t="n">
+      <c r="G8" s="8" t="n">
         <f aca="false">E8*F8</f>
         <v>0.7</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="C9" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="C9" s="16" t="s">
+      <c r="D9" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="D9" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="E9" s="11" t="n">
+      <c r="E9" s="6" t="n">
         <v>1</v>
       </c>
       <c r="F9" s="17" t="n">
         <v>1.34</v>
       </c>
-      <c r="G9" s="13" t="n">
+      <c r="G9" s="8" t="n">
         <f aca="false">E9*F9</f>
         <v>1.34</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="C10" s="16" t="s">
+      <c r="D10" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="D10" s="15" t="s">
-        <v>30</v>
-      </c>
-      <c r="E10" s="11" t="n">
+      <c r="E10" s="6" t="n">
         <v>2</v>
       </c>
       <c r="F10" s="17" t="n">
         <v>0.6</v>
       </c>
-      <c r="G10" s="13" t="n">
+      <c r="G10" s="8" t="n">
         <f aca="false">E10*F10</f>
         <v>1.2</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="18" t="s">
+      <c r="B11" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="C11" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="C11" s="19" t="s">
+      <c r="D11" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="D11" s="18" t="s">
-        <v>33</v>
-      </c>
       <c r="E11" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="F11" s="20" t="n">
+      <c r="F11" s="17" t="n">
         <v>0.49</v>
       </c>
       <c r="G11" s="8" t="n">
@@ -1068,783 +961,769 @@
     </row>
     <row r="12" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="C12" s="16" t="s">
         <v>34</v>
       </c>
-      <c r="C12" s="16" t="s">
+      <c r="D12" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="D12" s="15" t="s">
-        <v>36</v>
-      </c>
-      <c r="E12" s="11" t="n">
+      <c r="E12" s="6" t="n">
         <v>1</v>
       </c>
       <c r="F12" s="17" t="n">
         <v>0.84</v>
       </c>
-      <c r="G12" s="13" t="n">
+      <c r="G12" s="8" t="n">
         <f aca="false">E12*F12</f>
         <v>0.84</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="C13" s="16" t="s">
         <v>37</v>
       </c>
-      <c r="C13" s="16" t="s">
+      <c r="D13" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="D13" s="15" t="s">
-        <v>39</v>
-      </c>
-      <c r="E13" s="11" t="n">
+      <c r="E13" s="6" t="n">
         <v>1</v>
       </c>
       <c r="F13" s="17" t="n">
         <v>0.31</v>
       </c>
-      <c r="G13" s="13" t="n">
+      <c r="G13" s="8" t="n">
         <f aca="false">E13*F13</f>
         <v>0.31</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="18" t="s">
+      <c r="B14" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="C14" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="C14" s="21" t="s">
+      <c r="D14" s="15" t="s">
         <v>41</v>
-      </c>
-      <c r="D14" s="18" t="s">
-        <v>42</v>
       </c>
       <c r="E14" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="F14" s="20" t="n">
+      <c r="F14" s="17" t="n">
         <v>1.61</v>
       </c>
-      <c r="G14" s="22" t="n">
+      <c r="G14" s="8" t="n">
         <f aca="false">F14*E14</f>
         <v>3.22</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B15" s="23"/>
-      <c r="C15" s="23"/>
-      <c r="D15" s="23"/>
-      <c r="E15" s="23"/>
-      <c r="F15" s="24"/>
-      <c r="G15" s="23"/>
-      <c r="I15" s="0"/>
+      <c r="B15" s="18"/>
+      <c r="C15" s="18"/>
+      <c r="D15" s="18"/>
+      <c r="E15" s="18"/>
+      <c r="F15" s="13"/>
+      <c r="G15" s="18"/>
     </row>
     <row r="16" customFormat="false" ht="14.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="C16" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="C16" s="16" t="s">
+      <c r="D16" s="15" t="s">
         <v>44</v>
       </c>
-      <c r="D16" s="15" t="s">
-        <v>45</v>
-      </c>
-      <c r="E16" s="11" t="n">
+      <c r="E16" s="6" t="n">
         <v>1</v>
       </c>
       <c r="F16" s="17" t="n">
         <v>2.46</v>
       </c>
-      <c r="G16" s="13" t="n">
+      <c r="G16" s="8" t="n">
         <f aca="false">E16*F16</f>
         <v>2.46</v>
       </c>
-      <c r="I16" s="25" t="s">
-        <v>46</v>
-      </c>
+      <c r="I16" s="19"/>
     </row>
     <row r="17" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="15" t="s">
+        <v>45</v>
+      </c>
+      <c r="C17" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="D17" s="15" t="s">
         <v>47</v>
       </c>
-      <c r="C17" s="16" t="s">
-        <v>48</v>
-      </c>
-      <c r="D17" s="15" t="s">
-        <v>49</v>
-      </c>
-      <c r="E17" s="11" t="n">
+      <c r="E17" s="6" t="n">
         <v>1</v>
       </c>
       <c r="F17" s="17" t="n">
         <v>1.15</v>
       </c>
-      <c r="G17" s="13" t="n">
+      <c r="G17" s="8" t="n">
         <f aca="false">E17*F17</f>
         <v>1.15</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="15" t="s">
+        <v>48</v>
+      </c>
+      <c r="C18" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="D18" s="15" t="s">
         <v>50</v>
       </c>
-      <c r="C18" s="16" t="s">
-        <v>51</v>
-      </c>
-      <c r="D18" s="15" t="s">
-        <v>52</v>
-      </c>
-      <c r="E18" s="11" t="n">
+      <c r="E18" s="6" t="n">
         <v>1</v>
       </c>
       <c r="F18" s="17" t="n">
         <v>0.29</v>
       </c>
-      <c r="G18" s="13" t="n">
+      <c r="G18" s="8" t="n">
         <f aca="false">E18*F18</f>
         <v>0.29</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="C19" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="D19" s="15" t="s">
         <v>53</v>
       </c>
-      <c r="C19" s="16" t="s">
-        <v>54</v>
-      </c>
-      <c r="D19" s="15" t="s">
-        <v>55</v>
-      </c>
-      <c r="E19" s="11" t="n">
+      <c r="E19" s="6" t="n">
         <v>2</v>
       </c>
       <c r="F19" s="17" t="n">
         <v>0.18</v>
       </c>
-      <c r="G19" s="13" t="n">
+      <c r="G19" s="8" t="n">
         <f aca="false">E19*F19</f>
         <v>0.36</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="15" t="s">
+        <v>54</v>
+      </c>
+      <c r="C20" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="D20" s="15" t="s">
         <v>56</v>
       </c>
-      <c r="C20" s="16" t="s">
-        <v>57</v>
-      </c>
-      <c r="D20" s="15" t="s">
-        <v>58</v>
-      </c>
-      <c r="E20" s="11" t="n">
+      <c r="E20" s="6" t="n">
         <v>1</v>
       </c>
       <c r="F20" s="17" t="n">
         <v>0.31</v>
       </c>
-      <c r="G20" s="13" t="n">
+      <c r="G20" s="8" t="n">
         <f aca="false">E20*F20</f>
         <v>0.31</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="15"/>
-      <c r="C21" s="15"/>
-      <c r="D21" s="15"/>
-      <c r="E21" s="15"/>
-      <c r="F21" s="17"/>
-      <c r="G21" s="23"/>
+      <c r="B21" s="18"/>
+      <c r="C21" s="18"/>
+      <c r="D21" s="18"/>
+      <c r="E21" s="18"/>
+      <c r="F21" s="20"/>
+      <c r="G21" s="18"/>
     </row>
     <row r="22" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="C22" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="D22" s="15" t="s">
         <v>59</v>
       </c>
-      <c r="C22" s="16" t="s">
-        <v>60</v>
-      </c>
-      <c r="D22" s="15" t="s">
-        <v>61</v>
-      </c>
-      <c r="E22" s="11" t="n">
+      <c r="E22" s="6" t="n">
         <v>1</v>
       </c>
       <c r="F22" s="17" t="n">
-        <v>0.18</v>
-      </c>
-      <c r="G22" s="13" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G22" s="8" t="n">
         <f aca="false">E22*F22</f>
-        <v>0.18</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="15" t="s">
+        <v>60</v>
+      </c>
+      <c r="C23" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="D23" s="15" t="s">
         <v>62</v>
       </c>
-      <c r="C23" s="16" t="s">
-        <v>63</v>
-      </c>
-      <c r="D23" s="15" t="s">
-        <v>64</v>
-      </c>
-      <c r="E23" s="11" t="n">
+      <c r="E23" s="6" t="n">
         <v>2</v>
       </c>
       <c r="F23" s="17" t="n">
         <v>0.18</v>
       </c>
-      <c r="G23" s="13" t="n">
+      <c r="G23" s="8" t="n">
         <f aca="false">E23*F23</f>
         <v>0.36</v>
       </c>
-      <c r="I23" s="26" t="s">
-        <v>65</v>
-      </c>
+      <c r="H23" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="I23" s="0"/>
     </row>
     <row r="24" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="C24" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="D24" s="15" t="s">
         <v>66</v>
       </c>
-      <c r="C24" s="16" t="s">
-        <v>67</v>
-      </c>
-      <c r="D24" s="15" t="s">
-        <v>68</v>
-      </c>
-      <c r="E24" s="11" t="n">
+      <c r="E24" s="6" t="n">
         <v>1</v>
       </c>
       <c r="F24" s="17" t="n">
         <v>0.86</v>
       </c>
-      <c r="G24" s="13" t="n">
+      <c r="G24" s="8" t="n">
         <f aca="false">E24*F24</f>
         <v>0.86</v>
       </c>
-      <c r="I24" s="1" t="s">
-        <v>65</v>
-      </c>
+      <c r="H24" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="I24" s="0"/>
     </row>
     <row r="25" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="C25" s="16" t="s">
+        <v>68</v>
+      </c>
+      <c r="D25" s="15" t="s">
         <v>69</v>
       </c>
-      <c r="C25" s="16" t="s">
-        <v>70</v>
-      </c>
-      <c r="D25" s="15" t="s">
-        <v>71</v>
-      </c>
-      <c r="E25" s="11" t="n">
+      <c r="E25" s="6" t="n">
         <v>1</v>
       </c>
       <c r="F25" s="17" t="n">
         <v>0.18</v>
       </c>
-      <c r="G25" s="13" t="n">
+      <c r="G25" s="8" t="n">
         <f aca="false">E25*F25</f>
         <v>0.18</v>
       </c>
+      <c r="H25" s="1"/>
+      <c r="I25" s="0"/>
     </row>
     <row r="26" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="27" t="s">
+      <c r="B26" s="15" t="s">
+        <v>70</v>
+      </c>
+      <c r="C26" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="D26" s="15" t="s">
         <v>72</v>
       </c>
-      <c r="C26" s="28" t="s">
-        <v>73</v>
-      </c>
-      <c r="D26" s="27" t="s">
-        <v>74</v>
-      </c>
-      <c r="E26" s="29" t="n">
-        <v>1</v>
-      </c>
-      <c r="F26" s="30" t="n">
-        <v>0.57</v>
-      </c>
-      <c r="G26" s="31" t="n">
+      <c r="E26" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F26" s="17" t="n">
+        <v>1.23</v>
+      </c>
+      <c r="G26" s="8" t="n">
         <f aca="false">E26*F26</f>
-        <v>0.57</v>
-      </c>
-      <c r="H26" s="32"/>
-      <c r="I26" s="33" t="s">
-        <v>65</v>
-      </c>
-      <c r="J26" s="34" t="s">
-        <v>75</v>
-      </c>
+        <v>1.23</v>
+      </c>
+      <c r="H26" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="I26" s="0"/>
+      <c r="J26" s="14"/>
     </row>
     <row r="27" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="15" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="C27" s="16" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="D27" s="15" t="s">
-        <v>78</v>
-      </c>
-      <c r="E27" s="11" t="n">
+        <v>75</v>
+      </c>
+      <c r="E27" s="6" t="n">
         <v>1</v>
       </c>
       <c r="F27" s="17" t="n">
         <v>1.43</v>
       </c>
-      <c r="G27" s="13" t="n">
+      <c r="G27" s="8" t="n">
         <f aca="false">E27*F27</f>
         <v>1.43</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B28" s="15"/>
-      <c r="C28" s="15"/>
-      <c r="D28" s="15"/>
-      <c r="E28" s="15"/>
-      <c r="F28" s="35"/>
-      <c r="G28" s="23"/>
+      <c r="B28" s="18"/>
+      <c r="C28" s="18"/>
+      <c r="D28" s="18"/>
+      <c r="E28" s="18"/>
+      <c r="F28" s="21"/>
+      <c r="G28" s="18"/>
     </row>
     <row r="29" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="15" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="C29" s="16" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D29" s="15" t="s">
-        <v>81</v>
-      </c>
-      <c r="E29" s="11" t="n">
+        <v>78</v>
+      </c>
+      <c r="E29" s="6" t="n">
         <v>1</v>
       </c>
       <c r="F29" s="17" t="n">
         <v>0.18</v>
       </c>
-      <c r="G29" s="13" t="n">
+      <c r="G29" s="8" t="n">
         <f aca="false">E29*F29</f>
         <v>0.18</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="15" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="C30" s="16" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="D30" s="15" t="s">
-        <v>84</v>
-      </c>
-      <c r="E30" s="11" t="n">
+        <v>81</v>
+      </c>
+      <c r="E30" s="6" t="n">
         <v>1</v>
       </c>
       <c r="F30" s="17" t="n">
         <v>0.18</v>
       </c>
-      <c r="G30" s="13" t="n">
+      <c r="G30" s="8" t="n">
         <f aca="false">E30*F30</f>
         <v>0.18</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="15" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C31" s="16" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D31" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="E31" s="11" t="n">
+        <v>84</v>
+      </c>
+      <c r="E31" s="6" t="n">
         <v>4</v>
       </c>
       <c r="F31" s="17" t="n">
         <v>0.18</v>
       </c>
-      <c r="G31" s="13" t="n">
+      <c r="G31" s="8" t="n">
         <f aca="false">E31*F31</f>
         <v>0.72</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="15" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="C32" s="16" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="D32" s="15" t="s">
-        <v>90</v>
-      </c>
-      <c r="E32" s="11" t="n">
+        <v>87</v>
+      </c>
+      <c r="E32" s="6" t="n">
         <v>2</v>
       </c>
       <c r="F32" s="17" t="n">
         <v>0.18</v>
       </c>
-      <c r="G32" s="13" t="n">
+      <c r="G32" s="8" t="n">
         <f aca="false">E32*F32</f>
         <v>0.36</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="15" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="C33" s="16" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="D33" s="15" t="s">
-        <v>93</v>
-      </c>
-      <c r="E33" s="11" t="n">
+        <v>90</v>
+      </c>
+      <c r="E33" s="6" t="n">
         <v>1</v>
       </c>
       <c r="F33" s="17" t="n">
         <v>0.6</v>
       </c>
-      <c r="G33" s="13" t="n">
+      <c r="G33" s="8" t="n">
         <f aca="false">E33*F33</f>
         <v>0.6</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="15" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="C34" s="16" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D34" s="15" t="s">
-        <v>96</v>
-      </c>
-      <c r="E34" s="11" t="n">
+        <v>93</v>
+      </c>
+      <c r="E34" s="6" t="n">
         <v>1</v>
       </c>
       <c r="F34" s="17" t="n">
         <v>0.18</v>
       </c>
-      <c r="G34" s="13" t="n">
+      <c r="G34" s="8" t="n">
         <f aca="false">E34*F34</f>
         <v>0.18</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="15" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="C35" s="16" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="D35" s="15" t="s">
-        <v>99</v>
-      </c>
-      <c r="E35" s="11" t="n">
+        <v>96</v>
+      </c>
+      <c r="E35" s="6" t="n">
         <v>1</v>
       </c>
       <c r="F35" s="17" t="n">
         <v>0.18</v>
       </c>
-      <c r="G35" s="13" t="n">
+      <c r="G35" s="8" t="n">
         <f aca="false">E35*F35</f>
         <v>0.18</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="15" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="C36" s="16" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="D36" s="15" t="s">
-        <v>102</v>
-      </c>
-      <c r="E36" s="11" t="n">
+        <v>99</v>
+      </c>
+      <c r="E36" s="6" t="n">
         <v>4</v>
       </c>
       <c r="F36" s="17" t="n">
         <v>0.18</v>
       </c>
-      <c r="G36" s="13" t="n">
+      <c r="G36" s="8" t="n">
         <f aca="false">E36*F36</f>
         <v>0.72</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="15" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="C37" s="16" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D37" s="15" t="s">
-        <v>105</v>
-      </c>
-      <c r="E37" s="11" t="n">
+        <v>102</v>
+      </c>
+      <c r="E37" s="6" t="n">
         <v>2</v>
       </c>
       <c r="F37" s="17" t="n">
         <v>0.18</v>
       </c>
-      <c r="G37" s="13" t="n">
+      <c r="G37" s="8" t="n">
         <f aca="false">E37*F37</f>
         <v>0.36</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="15" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="C38" s="16" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="D38" s="15" t="s">
-        <v>108</v>
-      </c>
-      <c r="E38" s="11" t="n">
+        <v>105</v>
+      </c>
+      <c r="E38" s="6" t="n">
         <v>1</v>
       </c>
       <c r="F38" s="17" t="n">
         <v>2.36</v>
       </c>
-      <c r="G38" s="13" t="n">
+      <c r="G38" s="8" t="n">
         <f aca="false">E38*F38</f>
         <v>2.36</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B39" s="15"/>
-      <c r="C39" s="15"/>
-      <c r="D39" s="15"/>
-      <c r="E39" s="15"/>
-      <c r="F39" s="23"/>
-      <c r="G39" s="23"/>
+      <c r="B39" s="18"/>
+      <c r="C39" s="18"/>
+      <c r="D39" s="18"/>
+      <c r="E39" s="18"/>
+      <c r="F39" s="18"/>
+      <c r="G39" s="18"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B40" s="15"/>
-      <c r="C40" s="15"/>
-      <c r="D40" s="15"/>
-      <c r="E40" s="15"/>
-      <c r="F40" s="23"/>
-      <c r="G40" s="23"/>
+      <c r="B40" s="18"/>
+      <c r="C40" s="18"/>
+      <c r="D40" s="18"/>
+      <c r="E40" s="18"/>
+      <c r="F40" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="G40" s="22" t="n">
+        <f aca="false">SUM(G3:G39)</f>
+        <v>28.01</v>
+      </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B41" s="15"/>
-      <c r="C41" s="15"/>
-      <c r="D41" s="15"/>
-      <c r="E41" s="15"/>
-      <c r="F41" s="35"/>
-      <c r="G41" s="23"/>
+      <c r="B41" s="18"/>
+      <c r="C41" s="18"/>
+      <c r="D41" s="18"/>
+      <c r="E41" s="18"/>
+      <c r="F41" s="21"/>
+      <c r="G41" s="18"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B42" s="15"/>
-      <c r="C42" s="15"/>
-      <c r="D42" s="15"/>
-      <c r="E42" s="15"/>
-      <c r="F42" s="35"/>
-      <c r="G42" s="23"/>
+      <c r="B42" s="18"/>
+      <c r="C42" s="18"/>
+      <c r="D42" s="18"/>
+      <c r="E42" s="18"/>
+      <c r="F42" s="21"/>
+      <c r="G42" s="18"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B43" s="15"/>
-      <c r="C43" s="15"/>
-      <c r="D43" s="15"/>
-      <c r="E43" s="15"/>
-      <c r="F43" s="35"/>
-      <c r="G43" s="23"/>
+      <c r="B43" s="18"/>
+      <c r="C43" s="18"/>
+      <c r="D43" s="18"/>
+      <c r="E43" s="18"/>
+      <c r="F43" s="21"/>
+      <c r="G43" s="18"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B44" s="15"/>
-      <c r="C44" s="15"/>
-      <c r="D44" s="15"/>
-      <c r="E44" s="15"/>
-      <c r="F44" s="35"/>
-      <c r="G44" s="23"/>
+      <c r="B44" s="18"/>
+      <c r="C44" s="18"/>
+      <c r="D44" s="18"/>
+      <c r="E44" s="18"/>
+      <c r="F44" s="21"/>
+      <c r="G44" s="18"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B45" s="15"/>
-      <c r="C45" s="15"/>
-      <c r="D45" s="15"/>
+      <c r="B45" s="18"/>
+      <c r="C45" s="18"/>
+      <c r="D45" s="18"/>
       <c r="E45" s="11"/>
-      <c r="F45" s="17"/>
-      <c r="G45" s="13" t="n">
-        <f aca="false">E45*F45</f>
-        <v>0</v>
-      </c>
+      <c r="F45" s="20"/>
+      <c r="G45" s="13"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B46" s="15"/>
-      <c r="C46" s="36" t="s">
-        <v>109</v>
-      </c>
-      <c r="D46" s="15"/>
+      <c r="B46" s="18"/>
+      <c r="C46" s="23"/>
+      <c r="D46" s="18"/>
       <c r="E46" s="11"/>
-      <c r="F46" s="17"/>
-      <c r="G46" s="13" t="n">
-        <f aca="false">E46*F46</f>
-        <v>0</v>
-      </c>
+      <c r="F46" s="20"/>
+      <c r="G46" s="13"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B47" s="15"/>
-      <c r="C47" s="15"/>
-      <c r="D47" s="15"/>
+      <c r="B47" s="18"/>
+      <c r="C47" s="18"/>
+      <c r="D47" s="18"/>
       <c r="E47" s="11"/>
-      <c r="F47" s="35"/>
-      <c r="G47" s="13" t="n">
-        <f aca="false">E47*F47</f>
-        <v>0</v>
-      </c>
+      <c r="F47" s="21"/>
+      <c r="G47" s="13"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B48" s="15"/>
-      <c r="C48" s="15"/>
-      <c r="D48" s="15"/>
-      <c r="E48" s="15"/>
-      <c r="F48" s="11" t="s">
-        <v>110</v>
-      </c>
-      <c r="G48" s="37" t="n">
-        <f aca="false">SUM(G3:G46)</f>
-        <v>27.33</v>
-      </c>
+      <c r="B48" s="18"/>
+      <c r="C48" s="18"/>
+      <c r="D48" s="18"/>
+      <c r="E48" s="18"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G49" s="15"/>
+      <c r="G49" s="18"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B50" s="15"/>
-      <c r="C50" s="15"/>
-      <c r="D50" s="15"/>
-      <c r="E50" s="15"/>
-      <c r="F50" s="15"/>
-      <c r="G50" s="15"/>
+      <c r="B50" s="18"/>
+      <c r="C50" s="18"/>
+      <c r="D50" s="18"/>
+      <c r="E50" s="18"/>
+      <c r="F50" s="18"/>
+      <c r="G50" s="18"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B51" s="15"/>
-      <c r="C51" s="15"/>
-      <c r="D51" s="15"/>
-      <c r="E51" s="15"/>
-      <c r="F51" s="15"/>
-      <c r="G51" s="15"/>
+      <c r="B51" s="18"/>
+      <c r="C51" s="18"/>
+      <c r="D51" s="18"/>
+      <c r="E51" s="18"/>
+      <c r="F51" s="18"/>
+      <c r="G51" s="18"/>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B52" s="15"/>
-      <c r="C52" s="15"/>
-      <c r="D52" s="15"/>
-      <c r="E52" s="15"/>
-      <c r="F52" s="15"/>
-      <c r="G52" s="15"/>
+      <c r="B52" s="18"/>
+      <c r="C52" s="18"/>
+      <c r="D52" s="18"/>
+      <c r="E52" s="18"/>
+      <c r="F52" s="18"/>
+      <c r="G52" s="18"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B53" s="15"/>
-      <c r="C53" s="15"/>
-      <c r="D53" s="15"/>
-      <c r="E53" s="15"/>
-      <c r="F53" s="15"/>
-      <c r="G53" s="15"/>
+      <c r="B53" s="18"/>
+      <c r="C53" s="18"/>
+      <c r="D53" s="18"/>
+      <c r="E53" s="18"/>
+      <c r="F53" s="18"/>
+      <c r="G53" s="18"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B54" s="15"/>
-      <c r="C54" s="15"/>
-      <c r="D54" s="15"/>
-      <c r="E54" s="15"/>
-      <c r="F54" s="15"/>
-      <c r="G54" s="15"/>
+      <c r="B54" s="18"/>
+      <c r="C54" s="18"/>
+      <c r="D54" s="18"/>
+      <c r="E54" s="18"/>
+      <c r="F54" s="18"/>
+      <c r="G54" s="18"/>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B55" s="15"/>
-      <c r="C55" s="15"/>
-      <c r="D55" s="15"/>
-      <c r="E55" s="15"/>
-      <c r="F55" s="15"/>
-      <c r="G55" s="15"/>
+      <c r="B55" s="18"/>
+      <c r="C55" s="18"/>
+      <c r="D55" s="18"/>
+      <c r="E55" s="18"/>
+      <c r="F55" s="18"/>
+      <c r="G55" s="18"/>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B56" s="15"/>
-      <c r="C56" s="15"/>
-      <c r="D56" s="15"/>
-      <c r="E56" s="15"/>
-      <c r="F56" s="15"/>
-      <c r="G56" s="15"/>
+      <c r="B56" s="18"/>
+      <c r="C56" s="18"/>
+      <c r="D56" s="18"/>
+      <c r="E56" s="18"/>
+      <c r="F56" s="18"/>
+      <c r="G56" s="18"/>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B57" s="15"/>
-      <c r="C57" s="15"/>
-      <c r="D57" s="15"/>
-      <c r="E57" s="15"/>
-      <c r="F57" s="15"/>
-      <c r="G57" s="15"/>
+      <c r="B57" s="18"/>
+      <c r="C57" s="18"/>
+      <c r="D57" s="18"/>
+      <c r="E57" s="18"/>
+      <c r="F57" s="18"/>
+      <c r="G57" s="18"/>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B58" s="15"/>
-      <c r="C58" s="15"/>
-      <c r="D58" s="15"/>
-      <c r="E58" s="15"/>
-      <c r="F58" s="15"/>
-      <c r="G58" s="15"/>
+      <c r="B58" s="18"/>
+      <c r="C58" s="18"/>
+      <c r="D58" s="18"/>
+      <c r="E58" s="18"/>
+      <c r="F58" s="18"/>
+      <c r="G58" s="18"/>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B59" s="15"/>
-      <c r="C59" s="15"/>
-      <c r="D59" s="15"/>
-      <c r="E59" s="15"/>
-      <c r="F59" s="15"/>
-      <c r="G59" s="15"/>
+      <c r="B59" s="18"/>
+      <c r="C59" s="18"/>
+      <c r="D59" s="18"/>
+      <c r="E59" s="18"/>
+      <c r="F59" s="18"/>
+      <c r="G59" s="18"/>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B60" s="15"/>
-      <c r="C60" s="15"/>
-      <c r="D60" s="15"/>
-      <c r="E60" s="15"/>
-      <c r="F60" s="15"/>
-      <c r="G60" s="15"/>
+      <c r="B60" s="18"/>
+      <c r="C60" s="18"/>
+      <c r="D60" s="18"/>
+      <c r="E60" s="18"/>
+      <c r="F60" s="18"/>
+      <c r="G60" s="18"/>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B61" s="15"/>
-      <c r="C61" s="15"/>
-      <c r="D61" s="15"/>
-      <c r="E61" s="15"/>
-      <c r="F61" s="15"/>
-      <c r="G61" s="15"/>
+      <c r="B61" s="18"/>
+      <c r="C61" s="18"/>
+      <c r="D61" s="18"/>
+      <c r="E61" s="18"/>
+      <c r="F61" s="18"/>
+      <c r="G61" s="18"/>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B62" s="15"/>
-      <c r="C62" s="15"/>
-      <c r="D62" s="15"/>
-      <c r="E62" s="15"/>
-      <c r="F62" s="15"/>
-      <c r="G62" s="15"/>
+      <c r="B62" s="18"/>
+      <c r="C62" s="18"/>
+      <c r="D62" s="18"/>
+      <c r="E62" s="18"/>
+      <c r="F62" s="18"/>
+      <c r="G62" s="18"/>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B63" s="15"/>
-      <c r="C63" s="15"/>
-      <c r="D63" s="15"/>
-      <c r="E63" s="15"/>
-      <c r="F63" s="15"/>
-      <c r="G63" s="15"/>
+      <c r="B63" s="18"/>
+      <c r="C63" s="18"/>
+      <c r="D63" s="18"/>
+      <c r="E63" s="18"/>
+      <c r="F63" s="18"/>
+      <c r="G63" s="18"/>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B64" s="15"/>
-      <c r="C64" s="15"/>
-      <c r="D64" s="15"/>
-      <c r="E64" s="15"/>
-      <c r="F64" s="15"/>
-      <c r="G64" s="15"/>
+      <c r="B64" s="18"/>
+      <c r="C64" s="18"/>
+      <c r="D64" s="18"/>
+      <c r="E64" s="18"/>
+      <c r="F64" s="18"/>
+      <c r="G64" s="18"/>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B65" s="15"/>
-      <c r="C65" s="15"/>
-      <c r="D65" s="15"/>
-      <c r="E65" s="15"/>
-      <c r="F65" s="15"/>
-      <c r="G65" s="15"/>
+      <c r="B65" s="18"/>
+      <c r="C65" s="18"/>
+      <c r="D65" s="18"/>
+      <c r="E65" s="18"/>
+      <c r="F65" s="18"/>
+      <c r="G65" s="18"/>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B66" s="15"/>
-      <c r="C66" s="15"/>
-      <c r="D66" s="15"/>
-      <c r="E66" s="15"/>
-      <c r="F66" s="15"/>
-      <c r="G66" s="15"/>
+      <c r="B66" s="18"/>
+      <c r="C66" s="18"/>
+      <c r="D66" s="18"/>
+      <c r="E66" s="18"/>
+      <c r="F66" s="18"/>
+      <c r="G66" s="18"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -1859,17 +1738,17 @@
     <hyperlink ref="C11" r:id="rId9" display="https://www.digikey.co.nz/en/products/detail/te-connectivity-alcoswitch-switches/1-1825027-1/1632544 "/>
     <hyperlink ref="C12" r:id="rId10" display="https://www.digikey.co.nz/en/products/detail/sunled/XZCM2MOK54WA-1VF/15761908 "/>
     <hyperlink ref="C13" r:id="rId11" display="https://www.digikey.co.nz/en/products/detail/ams-osram-ag/LW-Q98G-01-R2T1-3K6L-1-5-R18/21556497 "/>
-    <hyperlink ref="C14" r:id="rId12" display="https://www.digikey.co.nz/en/products/detail/w%C3%BCrth-elektronik/61302011821/16608603"/>
+    <hyperlink ref="C14" r:id="rId12" display="https://www.digikey.co.nz/en/products/detail/w%C3%BCrth-elektronik/61302011821/16608603 "/>
     <hyperlink ref="C16" r:id="rId13" display="https://www.digikey.co.nz/en/products/detail/onsemi/FQD8P10TM/1054070 "/>
     <hyperlink ref="C17" r:id="rId14" display="https://www.digikey.co.nz/en/products/detail/diodes-incorporated/DMP3056L-7/5126843 "/>
     <hyperlink ref="C18" r:id="rId15" display="https://www.digikey.co.nz/en/products/detail/nexperia-usa-inc/NX138BKR/5981270 "/>
     <hyperlink ref="C19" r:id="rId16" display="https://www.digikey.co.nz/en/products/detail/shenzhen-slkormicro-semicon-co-ltd/SLMT320V3CN/29782446 "/>
     <hyperlink ref="C20" r:id="rId17" display="https://www.digikey.co.nz/en/products/detail/onsemi/MM3Z24VT1G/661665 "/>
-    <hyperlink ref="C22" r:id="rId18" display="https://www.digikey.co.nz/en/products/detail/w%C3%BCrth-elektronik/860010672004/5726903"/>
+    <hyperlink ref="C22" r:id="rId18" display="https://www.digikey.co.nz/en/products/detail/w%C3%BCrth-elektronik/860010572005/5726976"/>
     <hyperlink ref="C23" r:id="rId19" display="https://www.digikey.co.nz/en/products/detail/samsung-electro-mechanics/CL21B104KBCNNNC/3886661 "/>
-    <hyperlink ref="C24" r:id="rId20" display="https://www.digikey.co.nz/en/products/detail/tdk/C2012X5R1V106K125AC/3951654 "/>
+    <hyperlink ref="C24" r:id="rId20" display="https://www.digikey.co.nz/en/products/detail/tdk/C2012X5R1V106K085AC/3956083"/>
     <hyperlink ref="C25" r:id="rId21" display="https://www.digikey.co.nz/en/products/detail/murata-electronics/GCM1885C2A470JA16J/2591757 "/>
-    <hyperlink ref="C26" r:id="rId22" display="https://www.digikey.co.nz/en/products/detail/taiyo-yuden/JMK212BBJ476MG-T/4970731 "/>
+    <hyperlink ref="C26" r:id="rId22" display="https://www.digikey.co.nz/en/products/detail/tdk/C2012X5R0J476M125AC/2443465"/>
     <hyperlink ref="C27" r:id="rId23" display="https://www.digikey.co.nz/en/products/detail/tdk/SLF7045T-6R8M1R7-PF/755381 "/>
     <hyperlink ref="C29" r:id="rId24" display="https://www.digikey.co.nz/en/products/detail/bourns-inc/CR0805-FX-3012ELF/3784840 "/>
     <hyperlink ref="C30" r:id="rId25" display="https://www.digikey.co.nz/en/products/detail/bourns-inc/CR0805-FX-1583ELF/3784668 "/>

</xml_diff>

<commit_message>
Marking off parts for order
</commit_message>
<xml_diff>
--- a/Schematics & PCB/parts_order.xlsx
+++ b/Schematics & PCB/parts_order.xlsx
@@ -409,12 +409,18 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF70AFF2"/>
+        <bgColor rgb="FF99CCFF"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -457,7 +463,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="26">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -478,7 +484,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -486,11 +496,11 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -522,11 +532,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -581,7 +595,7 @@
       <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FFAFD095"/>
       <rgbColor rgb="FF808080"/>
-      <rgbColor rgb="FF9999FF"/>
+      <rgbColor rgb="FF70AFF2"/>
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FFFFFFCC"/>
       <rgbColor rgb="FFCCFFFF"/>
@@ -744,7 +758,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="102.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="34.4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="10.06"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="14.65"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="14.65"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="10.43"/>
   </cols>
   <sheetData>
@@ -775,16 +789,16 @@
       <c r="C3" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F3" s="7" t="n">
+      <c r="E3" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" s="8" t="n">
         <v>1.76</v>
       </c>
-      <c r="G3" s="8" t="n">
+      <c r="G3" s="9" t="n">
         <f aca="false">E3*F3</f>
         <v>1.76</v>
       </c>
@@ -796,934 +810,929 @@
       <c r="C4" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="E4" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F4" s="7" t="n">
+      <c r="E4" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" s="8" t="n">
         <v>2.86</v>
       </c>
-      <c r="G4" s="8" t="n">
+      <c r="G4" s="9" t="n">
         <f aca="false">E4*F4</f>
         <v>2.86</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="9" t="s">
+      <c r="B5" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="C5" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="D5" s="9" t="s">
+      <c r="D5" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="E5" s="11" t="n">
+      <c r="E5" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="F5" s="12" t="n">
+      <c r="F5" s="13" t="n">
         <v>14.04</v>
       </c>
-      <c r="G5" s="13" t="n">
+      <c r="G5" s="14" t="n">
         <f aca="false">E5*F5</f>
         <v>0</v>
       </c>
-      <c r="H5" s="14"/>
+      <c r="H5" s="15"/>
     </row>
     <row r="6" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="C6" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="9" t="s">
+      <c r="D6" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="E6" s="11" t="n">
+      <c r="E6" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="F6" s="12" t="n">
+      <c r="F6" s="13" t="n">
         <v>14.04</v>
       </c>
-      <c r="G6" s="13" t="n">
+      <c r="G6" s="14" t="n">
         <f aca="false">E6*F6</f>
         <v>0</v>
       </c>
-      <c r="H6" s="14"/>
+      <c r="H6" s="15"/>
     </row>
     <row r="7" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="15" t="s">
+      <c r="B7" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="16" t="s">
+      <c r="C7" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="D7" s="15" t="s">
+      <c r="D7" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="E7" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F7" s="17" t="n">
+      <c r="E7" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" s="19" t="n">
         <v>0.62</v>
       </c>
-      <c r="G7" s="8" t="n">
+      <c r="G7" s="9" t="n">
         <f aca="false">E7*F7</f>
         <v>0.62</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="15" t="s">
+      <c r="B8" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="C8" s="16" t="s">
+      <c r="C8" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="D8" s="15" t="s">
+      <c r="D8" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="E8" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F8" s="17" t="n">
+      <c r="E8" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" s="19" t="n">
         <v>0.7</v>
       </c>
-      <c r="G8" s="8" t="n">
+      <c r="G8" s="9" t="n">
         <f aca="false">E8*F8</f>
         <v>0.7</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="15" t="s">
+      <c r="B9" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="C9" s="16" t="s">
+      <c r="C9" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="D9" s="15" t="s">
+      <c r="D9" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="E9" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F9" s="17" t="n">
+      <c r="E9" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" s="19" t="n">
         <v>1.34</v>
       </c>
-      <c r="G9" s="8" t="n">
+      <c r="G9" s="9" t="n">
         <f aca="false">E9*F9</f>
         <v>1.34</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="15" t="s">
+      <c r="B10" s="16" t="s">
         <v>27</v>
       </c>
-      <c r="C10" s="16" t="s">
+      <c r="C10" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="D10" s="15" t="s">
+      <c r="D10" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="E10" s="6" t="n">
+      <c r="E10" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="F10" s="17" t="n">
+      <c r="F10" s="19" t="n">
         <v>0.6</v>
       </c>
-      <c r="G10" s="8" t="n">
+      <c r="G10" s="9" t="n">
         <f aca="false">E10*F10</f>
         <v>1.2</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="15" t="s">
+      <c r="B11" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="C11" s="16" t="s">
+      <c r="C11" s="17" t="s">
         <v>31</v>
       </c>
-      <c r="D11" s="15" t="s">
+      <c r="D11" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="E11" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F11" s="17" t="n">
+      <c r="E11" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" s="19" t="n">
         <v>0.49</v>
       </c>
-      <c r="G11" s="8" t="n">
+      <c r="G11" s="9" t="n">
         <f aca="false">E11*F11</f>
         <v>0.49</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="15" t="s">
+      <c r="B12" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="C12" s="16" t="s">
+      <c r="C12" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="D12" s="15" t="s">
+      <c r="D12" s="18" t="s">
         <v>35</v>
       </c>
-      <c r="E12" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F12" s="17" t="n">
+      <c r="E12" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="19" t="n">
         <v>0.84</v>
       </c>
-      <c r="G12" s="8" t="n">
+      <c r="G12" s="9" t="n">
         <f aca="false">E12*F12</f>
         <v>0.84</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="15" t="s">
+      <c r="B13" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="C13" s="16" t="s">
+      <c r="C13" s="17" t="s">
         <v>37</v>
       </c>
-      <c r="D13" s="15" t="s">
+      <c r="D13" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="E13" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F13" s="17" t="n">
+      <c r="E13" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" s="19" t="n">
         <v>0.31</v>
       </c>
-      <c r="G13" s="8" t="n">
+      <c r="G13" s="9" t="n">
         <f aca="false">E13*F13</f>
         <v>0.31</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="15" t="s">
+      <c r="B14" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="C14" s="16" t="s">
+      <c r="C14" s="17" t="s">
         <v>40</v>
       </c>
-      <c r="D14" s="15" t="s">
+      <c r="D14" s="18" t="s">
         <v>41</v>
       </c>
-      <c r="E14" s="6" t="n">
+      <c r="E14" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="F14" s="17" t="n">
+      <c r="F14" s="19" t="n">
         <v>1.61</v>
       </c>
-      <c r="G14" s="8" t="n">
+      <c r="G14" s="9" t="n">
         <f aca="false">F14*E14</f>
         <v>3.22</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B15" s="18"/>
-      <c r="C15" s="18"/>
-      <c r="D15" s="18"/>
-      <c r="E15" s="18"/>
-      <c r="F15" s="13"/>
-      <c r="G15" s="18"/>
+      <c r="B15" s="20"/>
+      <c r="C15" s="20"/>
+      <c r="D15" s="20"/>
+      <c r="E15" s="20"/>
+      <c r="F15" s="14"/>
+      <c r="G15" s="20"/>
     </row>
     <row r="16" customFormat="false" ht="14.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B16" s="15" t="s">
+      <c r="B16" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="C16" s="16" t="s">
+      <c r="C16" s="17" t="s">
         <v>43</v>
       </c>
-      <c r="D16" s="15" t="s">
+      <c r="D16" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="E16" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F16" s="17" t="n">
+      <c r="E16" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" s="19" t="n">
         <v>2.46</v>
       </c>
-      <c r="G16" s="8" t="n">
+      <c r="G16" s="9" t="n">
         <f aca="false">E16*F16</f>
         <v>2.46</v>
       </c>
-      <c r="I16" s="19"/>
+      <c r="I16" s="21"/>
     </row>
     <row r="17" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="15" t="s">
+      <c r="B17" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="C17" s="16" t="s">
+      <c r="C17" s="17" t="s">
         <v>46</v>
       </c>
-      <c r="D17" s="15" t="s">
+      <c r="D17" s="18" t="s">
         <v>47</v>
       </c>
-      <c r="E17" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F17" s="17" t="n">
+      <c r="E17" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" s="19" t="n">
         <v>1.15</v>
       </c>
-      <c r="G17" s="8" t="n">
+      <c r="G17" s="9" t="n">
         <f aca="false">E17*F17</f>
         <v>1.15</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="15" t="s">
+      <c r="B18" s="16" t="s">
         <v>48</v>
       </c>
-      <c r="C18" s="16" t="s">
+      <c r="C18" s="17" t="s">
         <v>49</v>
       </c>
-      <c r="D18" s="15" t="s">
+      <c r="D18" s="18" t="s">
         <v>50</v>
       </c>
-      <c r="E18" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F18" s="17" t="n">
+      <c r="E18" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" s="19" t="n">
         <v>0.29</v>
       </c>
-      <c r="G18" s="8" t="n">
+      <c r="G18" s="9" t="n">
         <f aca="false">E18*F18</f>
         <v>0.29</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="15" t="s">
+      <c r="B19" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="C19" s="16" t="s">
+      <c r="C19" s="17" t="s">
         <v>52</v>
       </c>
-      <c r="D19" s="15" t="s">
+      <c r="D19" s="18" t="s">
         <v>53</v>
       </c>
-      <c r="E19" s="6" t="n">
+      <c r="E19" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="F19" s="17" t="n">
+      <c r="F19" s="19" t="n">
         <v>0.18</v>
       </c>
-      <c r="G19" s="8" t="n">
+      <c r="G19" s="9" t="n">
         <f aca="false">E19*F19</f>
         <v>0.36</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="15" t="s">
+      <c r="B20" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="C20" s="16" t="s">
+      <c r="C20" s="17" t="s">
         <v>55</v>
       </c>
-      <c r="D20" s="15" t="s">
+      <c r="D20" s="18" t="s">
         <v>56</v>
       </c>
-      <c r="E20" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F20" s="17" t="n">
+      <c r="E20" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F20" s="19" t="n">
         <v>0.31</v>
       </c>
-      <c r="G20" s="8" t="n">
+      <c r="G20" s="9" t="n">
         <f aca="false">E20*F20</f>
         <v>0.31</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="18"/>
-      <c r="C21" s="18"/>
-      <c r="D21" s="18"/>
-      <c r="E21" s="18"/>
-      <c r="F21" s="20"/>
-      <c r="G21" s="18"/>
+      <c r="B21" s="20"/>
+      <c r="C21" s="20"/>
+      <c r="D21" s="20"/>
+      <c r="E21" s="20"/>
+      <c r="F21" s="22"/>
+      <c r="G21" s="20"/>
     </row>
     <row r="22" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="15" t="s">
+      <c r="B22" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="C22" s="16" t="s">
+      <c r="C22" s="17" t="s">
         <v>58</v>
       </c>
-      <c r="D22" s="15" t="s">
+      <c r="D22" s="18" t="s">
         <v>59</v>
       </c>
-      <c r="E22" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F22" s="17" t="n">
+      <c r="E22" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F22" s="19" t="n">
         <v>0.2</v>
       </c>
-      <c r="G22" s="8" t="n">
+      <c r="G22" s="9" t="n">
         <f aca="false">E22*F22</f>
         <v>0.2</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="15" t="s">
+      <c r="B23" s="16" t="s">
         <v>60</v>
       </c>
-      <c r="C23" s="16" t="s">
+      <c r="C23" s="17" t="s">
         <v>61</v>
       </c>
-      <c r="D23" s="15" t="s">
+      <c r="D23" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="E23" s="6" t="n">
+      <c r="E23" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="F23" s="17" t="n">
+      <c r="F23" s="19" t="n">
         <v>0.18</v>
       </c>
-      <c r="G23" s="8" t="n">
+      <c r="G23" s="9" t="n">
         <f aca="false">E23*F23</f>
         <v>0.36</v>
       </c>
       <c r="H23" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="I23" s="0"/>
     </row>
     <row r="24" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="15" t="s">
+      <c r="B24" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="C24" s="16" t="s">
+      <c r="C24" s="17" t="s">
         <v>65</v>
       </c>
-      <c r="D24" s="15" t="s">
+      <c r="D24" s="18" t="s">
         <v>66</v>
       </c>
-      <c r="E24" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F24" s="17" t="n">
+      <c r="E24" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F24" s="19" t="n">
         <v>0.86</v>
       </c>
-      <c r="G24" s="8" t="n">
+      <c r="G24" s="9" t="n">
         <f aca="false">E24*F24</f>
         <v>0.86</v>
       </c>
       <c r="H24" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="I24" s="0"/>
     </row>
     <row r="25" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="15" t="s">
+      <c r="B25" s="16" t="s">
         <v>67</v>
       </c>
-      <c r="C25" s="16" t="s">
+      <c r="C25" s="17" t="s">
         <v>68</v>
       </c>
-      <c r="D25" s="15" t="s">
+      <c r="D25" s="18" t="s">
         <v>69</v>
       </c>
-      <c r="E25" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F25" s="17" t="n">
+      <c r="E25" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F25" s="19" t="n">
         <v>0.18</v>
       </c>
-      <c r="G25" s="8" t="n">
+      <c r="G25" s="9" t="n">
         <f aca="false">E25*F25</f>
         <v>0.18</v>
       </c>
-      <c r="H25" s="1"/>
-      <c r="I25" s="0"/>
     </row>
     <row r="26" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="15" t="s">
+      <c r="B26" s="16" t="s">
         <v>70</v>
       </c>
-      <c r="C26" s="16" t="s">
+      <c r="C26" s="17" t="s">
         <v>71</v>
       </c>
-      <c r="D26" s="15" t="s">
+      <c r="D26" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="E26" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F26" s="17" t="n">
+      <c r="E26" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F26" s="19" t="n">
         <v>1.23</v>
       </c>
-      <c r="G26" s="8" t="n">
+      <c r="G26" s="9" t="n">
         <f aca="false">E26*F26</f>
         <v>1.23</v>
       </c>
       <c r="H26" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="I26" s="0"/>
-      <c r="J26" s="14"/>
+      <c r="J26" s="15"/>
     </row>
     <row r="27" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="15" t="s">
+      <c r="B27" s="16" t="s">
         <v>73</v>
       </c>
-      <c r="C27" s="16" t="s">
+      <c r="C27" s="17" t="s">
         <v>74</v>
       </c>
-      <c r="D27" s="15" t="s">
+      <c r="D27" s="18" t="s">
         <v>75</v>
       </c>
-      <c r="E27" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F27" s="17" t="n">
+      <c r="E27" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F27" s="19" t="n">
         <v>1.43</v>
       </c>
-      <c r="G27" s="8" t="n">
+      <c r="G27" s="9" t="n">
         <f aca="false">E27*F27</f>
         <v>1.43</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B28" s="18"/>
-      <c r="C28" s="18"/>
-      <c r="D28" s="18"/>
-      <c r="E28" s="18"/>
-      <c r="F28" s="21"/>
-      <c r="G28" s="18"/>
+      <c r="B28" s="20"/>
+      <c r="C28" s="20"/>
+      <c r="D28" s="20"/>
+      <c r="E28" s="20"/>
+      <c r="F28" s="23"/>
+      <c r="G28" s="20"/>
     </row>
     <row r="29" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B29" s="15" t="s">
+      <c r="B29" s="16" t="s">
         <v>76</v>
       </c>
-      <c r="C29" s="16" t="s">
+      <c r="C29" s="17" t="s">
         <v>77</v>
       </c>
-      <c r="D29" s="15" t="s">
+      <c r="D29" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="E29" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F29" s="17" t="n">
+      <c r="E29" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F29" s="19" t="n">
         <v>0.18</v>
       </c>
-      <c r="G29" s="8" t="n">
+      <c r="G29" s="9" t="n">
         <f aca="false">E29*F29</f>
         <v>0.18</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B30" s="15" t="s">
+      <c r="B30" s="16" t="s">
         <v>79</v>
       </c>
-      <c r="C30" s="16" t="s">
+      <c r="C30" s="17" t="s">
         <v>80</v>
       </c>
-      <c r="D30" s="15" t="s">
+      <c r="D30" s="18" t="s">
         <v>81</v>
       </c>
-      <c r="E30" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F30" s="17" t="n">
+      <c r="E30" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F30" s="19" t="n">
         <v>0.18</v>
       </c>
-      <c r="G30" s="8" t="n">
+      <c r="G30" s="9" t="n">
         <f aca="false">E30*F30</f>
         <v>0.18</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B31" s="15" t="s">
+      <c r="B31" s="16" t="s">
         <v>82</v>
       </c>
-      <c r="C31" s="16" t="s">
+      <c r="C31" s="17" t="s">
         <v>83</v>
       </c>
-      <c r="D31" s="15" t="s">
+      <c r="D31" s="18" t="s">
         <v>84</v>
       </c>
-      <c r="E31" s="6" t="n">
+      <c r="E31" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="F31" s="17" t="n">
+      <c r="F31" s="19" t="n">
         <v>0.18</v>
       </c>
-      <c r="G31" s="8" t="n">
+      <c r="G31" s="9" t="n">
         <f aca="false">E31*F31</f>
         <v>0.72</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B32" s="15" t="s">
+      <c r="B32" s="16" t="s">
         <v>85</v>
       </c>
-      <c r="C32" s="16" t="s">
+      <c r="C32" s="17" t="s">
         <v>86</v>
       </c>
-      <c r="D32" s="15" t="s">
+      <c r="D32" s="18" t="s">
         <v>87</v>
       </c>
-      <c r="E32" s="6" t="n">
+      <c r="E32" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="F32" s="17" t="n">
+      <c r="F32" s="19" t="n">
         <v>0.18</v>
       </c>
-      <c r="G32" s="8" t="n">
+      <c r="G32" s="9" t="n">
         <f aca="false">E32*F32</f>
         <v>0.36</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B33" s="15" t="s">
+      <c r="B33" s="16" t="s">
         <v>88</v>
       </c>
-      <c r="C33" s="16" t="s">
+      <c r="C33" s="17" t="s">
         <v>89</v>
       </c>
-      <c r="D33" s="15" t="s">
+      <c r="D33" s="18" t="s">
         <v>90</v>
       </c>
-      <c r="E33" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F33" s="17" t="n">
+      <c r="E33" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F33" s="19" t="n">
         <v>0.6</v>
       </c>
-      <c r="G33" s="8" t="n">
+      <c r="G33" s="9" t="n">
         <f aca="false">E33*F33</f>
         <v>0.6</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B34" s="15" t="s">
+      <c r="B34" s="16" t="s">
         <v>91</v>
       </c>
-      <c r="C34" s="16" t="s">
+      <c r="C34" s="17" t="s">
         <v>92</v>
       </c>
-      <c r="D34" s="15" t="s">
+      <c r="D34" s="18" t="s">
         <v>93</v>
       </c>
-      <c r="E34" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F34" s="17" t="n">
+      <c r="E34" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F34" s="19" t="n">
         <v>0.18</v>
       </c>
-      <c r="G34" s="8" t="n">
+      <c r="G34" s="9" t="n">
         <f aca="false">E34*F34</f>
         <v>0.18</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B35" s="15" t="s">
+      <c r="B35" s="16" t="s">
         <v>94</v>
       </c>
-      <c r="C35" s="16" t="s">
+      <c r="C35" s="17" t="s">
         <v>95</v>
       </c>
-      <c r="D35" s="15" t="s">
+      <c r="D35" s="18" t="s">
         <v>96</v>
       </c>
-      <c r="E35" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F35" s="17" t="n">
+      <c r="E35" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F35" s="19" t="n">
         <v>0.18</v>
       </c>
-      <c r="G35" s="8" t="n">
+      <c r="G35" s="9" t="n">
         <f aca="false">E35*F35</f>
         <v>0.18</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B36" s="15" t="s">
+      <c r="B36" s="16" t="s">
         <v>97</v>
       </c>
-      <c r="C36" s="16" t="s">
+      <c r="C36" s="17" t="s">
         <v>98</v>
       </c>
-      <c r="D36" s="15" t="s">
+      <c r="D36" s="18" t="s">
         <v>99</v>
       </c>
-      <c r="E36" s="6" t="n">
+      <c r="E36" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="F36" s="17" t="n">
+      <c r="F36" s="19" t="n">
         <v>0.18</v>
       </c>
-      <c r="G36" s="8" t="n">
+      <c r="G36" s="9" t="n">
         <f aca="false">E36*F36</f>
         <v>0.72</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B37" s="15" t="s">
+      <c r="B37" s="16" t="s">
         <v>100</v>
       </c>
-      <c r="C37" s="16" t="s">
+      <c r="C37" s="17" t="s">
         <v>101</v>
       </c>
-      <c r="D37" s="15" t="s">
+      <c r="D37" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="E37" s="6" t="n">
+      <c r="E37" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="F37" s="17" t="n">
+      <c r="F37" s="19" t="n">
         <v>0.18</v>
       </c>
-      <c r="G37" s="8" t="n">
+      <c r="G37" s="9" t="n">
         <f aca="false">E37*F37</f>
         <v>0.36</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B38" s="15" t="s">
+      <c r="B38" s="16" t="s">
         <v>103</v>
       </c>
-      <c r="C38" s="16" t="s">
+      <c r="C38" s="17" t="s">
         <v>104</v>
       </c>
-      <c r="D38" s="15" t="s">
+      <c r="D38" s="18" t="s">
         <v>105</v>
       </c>
-      <c r="E38" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F38" s="17" t="n">
+      <c r="E38" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F38" s="19" t="n">
         <v>2.36</v>
       </c>
-      <c r="G38" s="8" t="n">
+      <c r="G38" s="9" t="n">
         <f aca="false">E38*F38</f>
         <v>2.36</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B39" s="18"/>
-      <c r="C39" s="18"/>
-      <c r="D39" s="18"/>
-      <c r="E39" s="18"/>
-      <c r="F39" s="18"/>
-      <c r="G39" s="18"/>
+      <c r="B39" s="20"/>
+      <c r="C39" s="20"/>
+      <c r="D39" s="20"/>
+      <c r="E39" s="20"/>
+      <c r="F39" s="20"/>
+      <c r="G39" s="20"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B40" s="18"/>
-      <c r="C40" s="18"/>
-      <c r="D40" s="18"/>
-      <c r="E40" s="18"/>
-      <c r="F40" s="11" t="s">
+      <c r="B40" s="20"/>
+      <c r="C40" s="20"/>
+      <c r="D40" s="20"/>
+      <c r="E40" s="20"/>
+      <c r="F40" s="12" t="s">
         <v>106</v>
       </c>
-      <c r="G40" s="22" t="n">
+      <c r="G40" s="24" t="n">
         <f aca="false">SUM(G3:G39)</f>
         <v>28.01</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B41" s="18"/>
-      <c r="C41" s="18"/>
-      <c r="D41" s="18"/>
-      <c r="E41" s="18"/>
-      <c r="F41" s="21"/>
-      <c r="G41" s="18"/>
+      <c r="B41" s="20"/>
+      <c r="C41" s="20"/>
+      <c r="D41" s="20"/>
+      <c r="E41" s="20"/>
+      <c r="F41" s="23"/>
+      <c r="G41" s="20"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B42" s="18"/>
-      <c r="C42" s="18"/>
-      <c r="D42" s="18"/>
-      <c r="E42" s="18"/>
-      <c r="F42" s="21"/>
-      <c r="G42" s="18"/>
+      <c r="B42" s="20"/>
+      <c r="C42" s="20"/>
+      <c r="D42" s="20"/>
+      <c r="E42" s="20"/>
+      <c r="F42" s="23"/>
+      <c r="G42" s="20"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B43" s="18"/>
-      <c r="C43" s="18"/>
-      <c r="D43" s="18"/>
-      <c r="E43" s="18"/>
-      <c r="F43" s="21"/>
-      <c r="G43" s="18"/>
+      <c r="B43" s="20"/>
+      <c r="C43" s="20"/>
+      <c r="D43" s="20"/>
+      <c r="E43" s="20"/>
+      <c r="F43" s="23"/>
+      <c r="G43" s="20"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B44" s="18"/>
-      <c r="C44" s="18"/>
-      <c r="D44" s="18"/>
-      <c r="E44" s="18"/>
-      <c r="F44" s="21"/>
-      <c r="G44" s="18"/>
+      <c r="B44" s="20"/>
+      <c r="C44" s="20"/>
+      <c r="D44" s="20"/>
+      <c r="E44" s="20"/>
+      <c r="F44" s="23"/>
+      <c r="G44" s="20"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B45" s="18"/>
-      <c r="C45" s="18"/>
-      <c r="D45" s="18"/>
-      <c r="E45" s="11"/>
-      <c r="F45" s="20"/>
-      <c r="G45" s="13"/>
+      <c r="B45" s="20"/>
+      <c r="C45" s="20"/>
+      <c r="D45" s="20"/>
+      <c r="E45" s="12"/>
+      <c r="F45" s="22"/>
+      <c r="G45" s="14"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B46" s="18"/>
-      <c r="C46" s="23"/>
-      <c r="D46" s="18"/>
-      <c r="E46" s="11"/>
-      <c r="F46" s="20"/>
-      <c r="G46" s="13"/>
+      <c r="B46" s="20"/>
+      <c r="C46" s="25"/>
+      <c r="D46" s="20"/>
+      <c r="E46" s="12"/>
+      <c r="F46" s="22"/>
+      <c r="G46" s="14"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B47" s="18"/>
-      <c r="C47" s="18"/>
-      <c r="D47" s="18"/>
-      <c r="E47" s="11"/>
-      <c r="F47" s="21"/>
-      <c r="G47" s="13"/>
+      <c r="B47" s="20"/>
+      <c r="C47" s="20"/>
+      <c r="D47" s="20"/>
+      <c r="E47" s="12"/>
+      <c r="F47" s="23"/>
+      <c r="G47" s="14"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B48" s="18"/>
-      <c r="C48" s="18"/>
-      <c r="D48" s="18"/>
-      <c r="E48" s="18"/>
+      <c r="B48" s="20"/>
+      <c r="C48" s="20"/>
+      <c r="D48" s="20"/>
+      <c r="E48" s="20"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G49" s="18"/>
+      <c r="G49" s="20"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B50" s="18"/>
-      <c r="C50" s="18"/>
-      <c r="D50" s="18"/>
-      <c r="E50" s="18"/>
-      <c r="F50" s="18"/>
-      <c r="G50" s="18"/>
+      <c r="B50" s="20"/>
+      <c r="C50" s="20"/>
+      <c r="D50" s="20"/>
+      <c r="E50" s="20"/>
+      <c r="F50" s="20"/>
+      <c r="G50" s="20"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B51" s="18"/>
-      <c r="C51" s="18"/>
-      <c r="D51" s="18"/>
-      <c r="E51" s="18"/>
-      <c r="F51" s="18"/>
-      <c r="G51" s="18"/>
+      <c r="B51" s="20"/>
+      <c r="C51" s="20"/>
+      <c r="D51" s="20"/>
+      <c r="E51" s="20"/>
+      <c r="F51" s="20"/>
+      <c r="G51" s="20"/>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B52" s="18"/>
-      <c r="C52" s="18"/>
-      <c r="D52" s="18"/>
-      <c r="E52" s="18"/>
-      <c r="F52" s="18"/>
-      <c r="G52" s="18"/>
+      <c r="B52" s="20"/>
+      <c r="C52" s="20"/>
+      <c r="D52" s="20"/>
+      <c r="E52" s="20"/>
+      <c r="F52" s="20"/>
+      <c r="G52" s="20"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B53" s="18"/>
-      <c r="C53" s="18"/>
-      <c r="D53" s="18"/>
-      <c r="E53" s="18"/>
-      <c r="F53" s="18"/>
-      <c r="G53" s="18"/>
+      <c r="B53" s="20"/>
+      <c r="C53" s="20"/>
+      <c r="D53" s="20"/>
+      <c r="E53" s="20"/>
+      <c r="F53" s="20"/>
+      <c r="G53" s="20"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B54" s="18"/>
-      <c r="C54" s="18"/>
-      <c r="D54" s="18"/>
-      <c r="E54" s="18"/>
-      <c r="F54" s="18"/>
-      <c r="G54" s="18"/>
+      <c r="B54" s="20"/>
+      <c r="C54" s="20"/>
+      <c r="D54" s="20"/>
+      <c r="E54" s="20"/>
+      <c r="F54" s="20"/>
+      <c r="G54" s="20"/>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B55" s="18"/>
-      <c r="C55" s="18"/>
-      <c r="D55" s="18"/>
-      <c r="E55" s="18"/>
-      <c r="F55" s="18"/>
-      <c r="G55" s="18"/>
+      <c r="B55" s="20"/>
+      <c r="C55" s="20"/>
+      <c r="D55" s="20"/>
+      <c r="E55" s="20"/>
+      <c r="F55" s="20"/>
+      <c r="G55" s="20"/>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B56" s="18"/>
-      <c r="C56" s="18"/>
-      <c r="D56" s="18"/>
-      <c r="E56" s="18"/>
-      <c r="F56" s="18"/>
-      <c r="G56" s="18"/>
+      <c r="B56" s="20"/>
+      <c r="C56" s="20"/>
+      <c r="D56" s="20"/>
+      <c r="E56" s="20"/>
+      <c r="F56" s="20"/>
+      <c r="G56" s="20"/>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B57" s="18"/>
-      <c r="C57" s="18"/>
-      <c r="D57" s="18"/>
-      <c r="E57" s="18"/>
-      <c r="F57" s="18"/>
-      <c r="G57" s="18"/>
+      <c r="B57" s="20"/>
+      <c r="C57" s="20"/>
+      <c r="D57" s="20"/>
+      <c r="E57" s="20"/>
+      <c r="F57" s="20"/>
+      <c r="G57" s="20"/>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B58" s="18"/>
-      <c r="C58" s="18"/>
-      <c r="D58" s="18"/>
-      <c r="E58" s="18"/>
-      <c r="F58" s="18"/>
-      <c r="G58" s="18"/>
+      <c r="B58" s="20"/>
+      <c r="C58" s="20"/>
+      <c r="D58" s="20"/>
+      <c r="E58" s="20"/>
+      <c r="F58" s="20"/>
+      <c r="G58" s="20"/>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B59" s="18"/>
-      <c r="C59" s="18"/>
-      <c r="D59" s="18"/>
-      <c r="E59" s="18"/>
-      <c r="F59" s="18"/>
-      <c r="G59" s="18"/>
+      <c r="B59" s="20"/>
+      <c r="C59" s="20"/>
+      <c r="D59" s="20"/>
+      <c r="E59" s="20"/>
+      <c r="F59" s="20"/>
+      <c r="G59" s="20"/>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B60" s="18"/>
-      <c r="C60" s="18"/>
-      <c r="D60" s="18"/>
-      <c r="E60" s="18"/>
-      <c r="F60" s="18"/>
-      <c r="G60" s="18"/>
+      <c r="B60" s="20"/>
+      <c r="C60" s="20"/>
+      <c r="D60" s="20"/>
+      <c r="E60" s="20"/>
+      <c r="F60" s="20"/>
+      <c r="G60" s="20"/>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B61" s="18"/>
-      <c r="C61" s="18"/>
-      <c r="D61" s="18"/>
-      <c r="E61" s="18"/>
-      <c r="F61" s="18"/>
-      <c r="G61" s="18"/>
+      <c r="B61" s="20"/>
+      <c r="C61" s="20"/>
+      <c r="D61" s="20"/>
+      <c r="E61" s="20"/>
+      <c r="F61" s="20"/>
+      <c r="G61" s="20"/>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B62" s="18"/>
-      <c r="C62" s="18"/>
-      <c r="D62" s="18"/>
-      <c r="E62" s="18"/>
-      <c r="F62" s="18"/>
-      <c r="G62" s="18"/>
+      <c r="B62" s="20"/>
+      <c r="C62" s="20"/>
+      <c r="D62" s="20"/>
+      <c r="E62" s="20"/>
+      <c r="F62" s="20"/>
+      <c r="G62" s="20"/>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B63" s="18"/>
-      <c r="C63" s="18"/>
-      <c r="D63" s="18"/>
-      <c r="E63" s="18"/>
-      <c r="F63" s="18"/>
-      <c r="G63" s="18"/>
+      <c r="B63" s="20"/>
+      <c r="C63" s="20"/>
+      <c r="D63" s="20"/>
+      <c r="E63" s="20"/>
+      <c r="F63" s="20"/>
+      <c r="G63" s="20"/>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B64" s="18"/>
-      <c r="C64" s="18"/>
-      <c r="D64" s="18"/>
-      <c r="E64" s="18"/>
-      <c r="F64" s="18"/>
-      <c r="G64" s="18"/>
+      <c r="B64" s="20"/>
+      <c r="C64" s="20"/>
+      <c r="D64" s="20"/>
+      <c r="E64" s="20"/>
+      <c r="F64" s="20"/>
+      <c r="G64" s="20"/>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B65" s="18"/>
-      <c r="C65" s="18"/>
-      <c r="D65" s="18"/>
-      <c r="E65" s="18"/>
-      <c r="F65" s="18"/>
-      <c r="G65" s="18"/>
+      <c r="B65" s="20"/>
+      <c r="C65" s="20"/>
+      <c r="D65" s="20"/>
+      <c r="E65" s="20"/>
+      <c r="F65" s="20"/>
+      <c r="G65" s="20"/>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B66" s="18"/>
-      <c r="C66" s="18"/>
-      <c r="D66" s="18"/>
-      <c r="E66" s="18"/>
-      <c r="F66" s="18"/>
-      <c r="G66" s="18"/>
+      <c r="B66" s="20"/>
+      <c r="C66" s="20"/>
+      <c r="D66" s="20"/>
+      <c r="E66" s="20"/>
+      <c r="F66" s="20"/>
+      <c r="G66" s="20"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -1744,11 +1753,11 @@
     <hyperlink ref="C18" r:id="rId15" display="https://www.digikey.co.nz/en/products/detail/nexperia-usa-inc/NX138BKR/5981270 "/>
     <hyperlink ref="C19" r:id="rId16" display="https://www.digikey.co.nz/en/products/detail/shenzhen-slkormicro-semicon-co-ltd/SLMT320V3CN/29782446 "/>
     <hyperlink ref="C20" r:id="rId17" display="https://www.digikey.co.nz/en/products/detail/onsemi/MM3Z24VT1G/661665 "/>
-    <hyperlink ref="C22" r:id="rId18" display="https://www.digikey.co.nz/en/products/detail/w%C3%BCrth-elektronik/860010572005/5726976"/>
+    <hyperlink ref="C22" r:id="rId18" display="https://www.digikey.co.nz/en/products/detail/w%C3%BCrth-elektronik/860010572005/5726976 "/>
     <hyperlink ref="C23" r:id="rId19" display="https://www.digikey.co.nz/en/products/detail/samsung-electro-mechanics/CL21B104KBCNNNC/3886661 "/>
-    <hyperlink ref="C24" r:id="rId20" display="https://www.digikey.co.nz/en/products/detail/tdk/C2012X5R1V106K085AC/3956083"/>
+    <hyperlink ref="C24" r:id="rId20" display="https://www.digikey.co.nz/en/products/detail/tdk/C2012X5R1V106K085AC/3956083 "/>
     <hyperlink ref="C25" r:id="rId21" display="https://www.digikey.co.nz/en/products/detail/murata-electronics/GCM1885C2A470JA16J/2591757 "/>
-    <hyperlink ref="C26" r:id="rId22" display="https://www.digikey.co.nz/en/products/detail/tdk/C2012X5R0J476M125AC/2443465"/>
+    <hyperlink ref="C26" r:id="rId22" display="https://www.digikey.co.nz/en/products/detail/tdk/C2012X5R0J476M125AC/2443465 "/>
     <hyperlink ref="C27" r:id="rId23" display="https://www.digikey.co.nz/en/products/detail/tdk/SLF7045T-6R8M1R7-PF/755381 "/>
     <hyperlink ref="C29" r:id="rId24" display="https://www.digikey.co.nz/en/products/detail/bourns-inc/CR0805-FX-3012ELF/3784840 "/>
     <hyperlink ref="C30" r:id="rId25" display="https://www.digikey.co.nz/en/products/detail/bourns-inc/CR0805-FX-1583ELF/3784668 "/>

</xml_diff>